<commit_message>
Add 3 more promoters via awards angle (171 total)
Found via the Prémio Nacional do Imobiliário 2026 finalists list:
Violas Ferreira (Grupo HVF), Selicomi Portugal, Square Asset
Management. Also folds their finalist project into EastBanc
Portugal's existing entry (Anjos Urban Palace).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SRBJwGmSsYkTHKJbGCM5ca
</commit_message>
<xml_diff>
--- a/Lista_Contactos.xlsx
+++ b/Lista_Contactos.xlsx
@@ -203,8 +203,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Contactos" displayName="Contactos" ref="A1:J169" headerRowCount="1">
-  <autoFilter ref="A1:J169"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Contactos" displayName="Contactos" ref="A1:J172" headerRowCount="1">
+  <autoFilter ref="A1:J172"/>
   <tableColumns count="10">
     <tableColumn id="1" name="Nome da Empresa"/>
     <tableColumn id="2" name="Prioritario"/>
@@ -510,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J169"/>
+  <dimension ref="A1:J172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4316,7 +4316,7 @@
     <row r="86" ht="26" customHeight="1">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>Vomera Group</t>
+          <t>Violas Ferreira (Grupo HVF)</t>
         </is>
       </c>
       <c r="B86" s="4" t="inlineStr">
@@ -4326,77 +4326,81 @@
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>351 243 078 442</t>
+          <t>+351 227 340 823</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>Sérgio Santos (CEO/fundador, com Delphine Gerardo)</t>
+          <t>Tiago Violas Ferreira (líder do grupo)</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr"/>
       <c r="F86" s="2" t="inlineStr"/>
-      <c r="G86" s="2" t="inlineStr"/>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>info@violasferreira.com</t>
+        </is>
+      </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
+          <t>violasferreira.com</t>
+        </is>
+      </c>
+      <c r="I86" s="4" t="inlineStr">
+        <is>
+          <t>Espinho</t>
+        </is>
+      </c>
+      <c r="J86" s="4" t="inlineStr">
+        <is>
+          <t>Aveiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="26" customHeight="1">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>Vomera Group</t>
+        </is>
+      </c>
+      <c r="B87" s="4" t="inlineStr">
+        <is>
+          <t>Nao</t>
+        </is>
+      </c>
+      <c r="C87" s="4" t="inlineStr">
+        <is>
+          <t>351 243 078 442</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>Sérgio Santos (CEO/fundador, com Delphine Gerardo)</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr"/>
+      <c r="F87" s="2" t="inlineStr"/>
+      <c r="G87" s="2" t="inlineStr"/>
+      <c r="H87" s="2" t="inlineStr">
+        <is>
           <t>vomera.pt</t>
         </is>
       </c>
-      <c r="I86" s="4" t="inlineStr">
+      <c r="I87" s="4" t="inlineStr">
         <is>
           <t>Santarém</t>
         </is>
       </c>
-      <c r="J86" s="4" t="inlineStr">
+      <c r="J87" s="4" t="inlineStr">
         <is>
           <t>Santarém</t>
-        </is>
-      </c>
-    </row>
-    <row r="87" ht="26" customHeight="1">
-      <c r="A87" s="6" t="inlineStr">
-        <is>
-          <t>Alecrim Real Estate (Lince Capital)</t>
-        </is>
-      </c>
-      <c r="B87" s="7" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="C87" s="8" t="inlineStr"/>
-      <c r="D87" s="6" t="inlineStr">
-        <is>
-          <t>António Velho da Palma (CEO Alecrim RE)· CEO da holding Lince Capital é Vasco Pereira Coutinho</t>
-        </is>
-      </c>
-      <c r="E87" s="9" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/ant%C3%B3nio-velho-da-palma-82112282/</t>
-        </is>
-      </c>
-      <c r="F87" s="6" t="inlineStr"/>
-      <c r="G87" s="6" t="inlineStr"/>
-      <c r="H87" s="6" t="inlineStr">
-        <is>
-          <t>lince-capital.com</t>
-        </is>
-      </c>
-      <c r="I87" s="8" t="inlineStr">
-        <is>
-          <t>Lisboa</t>
-        </is>
-      </c>
-      <c r="J87" s="8" t="inlineStr">
-        <is>
-          <t>Lisboa</t>
         </is>
       </c>
     </row>
     <row r="88" ht="26" customHeight="1">
       <c r="A88" s="6" t="inlineStr">
         <is>
-          <t>VIZTA (ex-Nexity Portugal)</t>
+          <t>Alecrim Real Estate (Lince Capital)</t>
         </is>
       </c>
       <c r="B88" s="7" t="inlineStr">
@@ -4407,23 +4411,19 @@
       <c r="C88" s="8" t="inlineStr"/>
       <c r="D88" s="6" t="inlineStr">
         <is>
-          <t>Fernando Vasco Costa (CEO)</t>
+          <t>António Velho da Palma (CEO Alecrim RE)· CEO da holding Lince Capital é Vasco Pereira Coutinho</t>
         </is>
       </c>
       <c r="E88" s="9" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/fernando-vasco-costa/</t>
+          <t>https://www.linkedin.com/in/ant%C3%B3nio-velho-da-palma-82112282/</t>
         </is>
       </c>
       <c r="F88" s="6" t="inlineStr"/>
-      <c r="G88" s="6" t="inlineStr">
-        <is>
-          <t>privacidade@vizta.pt</t>
-        </is>
-      </c>
+      <c r="G88" s="6" t="inlineStr"/>
       <c r="H88" s="6" t="inlineStr">
         <is>
-          <t>vizta.pt</t>
+          <t>lince-capital.com</t>
         </is>
       </c>
       <c r="I88" s="8" t="inlineStr">
@@ -4440,7 +4440,7 @@
     <row r="89" ht="26" customHeight="1">
       <c r="A89" s="6" t="inlineStr">
         <is>
-          <t>Âncora Investments</t>
+          <t>VIZTA (ex-Nexity Portugal)</t>
         </is>
       </c>
       <c r="B89" s="7" t="inlineStr">
@@ -4451,40 +4451,40 @@
       <c r="C89" s="8" t="inlineStr"/>
       <c r="D89" s="6" t="inlineStr">
         <is>
-          <t>Elad Shachar e Tamir Luria (co-líderes/investidores)</t>
+          <t>Fernando Vasco Costa (CEO)</t>
         </is>
       </c>
       <c r="E89" s="9" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/tamir-luria/</t>
+          <t>https://www.linkedin.com/in/fernando-vasco-costa/</t>
         </is>
       </c>
       <c r="F89" s="6" t="inlineStr"/>
       <c r="G89" s="6" t="inlineStr">
         <is>
-          <t>info@ancora-inv.com</t>
+          <t>privacidade@vizta.pt</t>
         </is>
       </c>
       <c r="H89" s="6" t="inlineStr">
         <is>
-          <t>ancora-inv.com</t>
+          <t>vizta.pt</t>
         </is>
       </c>
       <c r="I89" s="8" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="J89" s="8" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Lisboa</t>
         </is>
       </c>
     </row>
     <row r="90" ht="26" customHeight="1">
       <c r="A90" s="6" t="inlineStr">
         <is>
-          <t>Década Paralela (Grupo Latitude, com a TPS)</t>
+          <t>Âncora Investments</t>
         </is>
       </c>
       <c r="B90" s="7" t="inlineStr">
@@ -4495,13 +4495,25 @@
       <c r="C90" s="8" t="inlineStr"/>
       <c r="D90" s="6" t="inlineStr">
         <is>
-          <t>Bruno Soares (CEO, família Soares/Latitude Capital)</t>
-        </is>
-      </c>
-      <c r="E90" s="6" t="inlineStr"/>
+          <t>Elad Shachar e Tamir Luria (co-líderes/investidores)</t>
+        </is>
+      </c>
+      <c r="E90" s="9" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/tamir-luria/</t>
+        </is>
+      </c>
       <c r="F90" s="6" t="inlineStr"/>
-      <c r="G90" s="6" t="inlineStr"/>
-      <c r="H90" s="6" t="inlineStr"/>
+      <c r="G90" s="6" t="inlineStr">
+        <is>
+          <t>info@ancora-inv.com</t>
+        </is>
+      </c>
+      <c r="H90" s="6" t="inlineStr">
+        <is>
+          <t>ancora-inv.com</t>
+        </is>
+      </c>
       <c r="I90" s="8" t="inlineStr">
         <is>
           <t>Porto</t>
@@ -4516,7 +4528,7 @@
     <row r="91" ht="26" customHeight="1">
       <c r="A91" s="6" t="inlineStr">
         <is>
-          <t>Frederico Ressano (promotor individual)</t>
+          <t>Década Paralela (Grupo Latitude, com a TPS)</t>
         </is>
       </c>
       <c r="B91" s="7" t="inlineStr">
@@ -4527,32 +4539,28 @@
       <c r="C91" s="8" t="inlineStr"/>
       <c r="D91" s="6" t="inlineStr">
         <is>
-          <t>Frederico Ressano</t>
+          <t>Bruno Soares (CEO, família Soares/Latitude Capital)</t>
         </is>
       </c>
       <c r="E91" s="6" t="inlineStr"/>
       <c r="F91" s="6" t="inlineStr"/>
       <c r="G91" s="6" t="inlineStr"/>
-      <c r="H91" s="6" t="inlineStr">
-        <is>
-          <t>theparkcascaisresidences.com</t>
-        </is>
-      </c>
+      <c r="H91" s="6" t="inlineStr"/>
       <c r="I91" s="8" t="inlineStr">
         <is>
-          <t>Cascais</t>
+          <t>Porto</t>
         </is>
       </c>
       <c r="J91" s="8" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Porto</t>
         </is>
       </c>
     </row>
     <row r="92" ht="26" customHeight="1">
       <c r="A92" s="6" t="inlineStr">
         <is>
-          <t>Fungepi (Grupo Novo Banco)</t>
+          <t>Frederico Ressano (promotor individual)</t>
         </is>
       </c>
       <c r="B92" s="7" t="inlineStr">
@@ -4561,14 +4569,22 @@
         </is>
       </c>
       <c r="C92" s="8" t="inlineStr"/>
-      <c r="D92" s="6" t="inlineStr"/>
+      <c r="D92" s="6" t="inlineStr">
+        <is>
+          <t>Frederico Ressano</t>
+        </is>
+      </c>
       <c r="E92" s="6" t="inlineStr"/>
       <c r="F92" s="6" t="inlineStr"/>
       <c r="G92" s="6" t="inlineStr"/>
-      <c r="H92" s="6" t="inlineStr"/>
+      <c r="H92" s="6" t="inlineStr">
+        <is>
+          <t>theparkcascaisresidences.com</t>
+        </is>
+      </c>
       <c r="I92" s="8" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Cascais</t>
         </is>
       </c>
       <c r="J92" s="8" t="inlineStr">
@@ -4580,7 +4596,7 @@
     <row r="93" ht="26" customHeight="1">
       <c r="A93" s="6" t="inlineStr">
         <is>
-          <t>Hines Portugal</t>
+          <t>Fungepi (Grupo Novo Banco)</t>
         </is>
       </c>
       <c r="B93" s="7" t="inlineStr">
@@ -4589,19 +4605,11 @@
         </is>
       </c>
       <c r="C93" s="8" t="inlineStr"/>
-      <c r="D93" s="6" t="inlineStr">
-        <is>
-          <t>Vanessa Gelado (Senior Managing Director, Head of Southern Europe)</t>
-        </is>
-      </c>
+      <c r="D93" s="6" t="inlineStr"/>
       <c r="E93" s="6" t="inlineStr"/>
       <c r="F93" s="6" t="inlineStr"/>
       <c r="G93" s="6" t="inlineStr"/>
-      <c r="H93" s="6" t="inlineStr">
-        <is>
-          <t>hines.com</t>
-        </is>
-      </c>
+      <c r="H93" s="6" t="inlineStr"/>
       <c r="I93" s="8" t="inlineStr">
         <is>
           <t>Lisboa</t>
@@ -4616,7 +4624,7 @@
     <row r="94" ht="26" customHeight="1">
       <c r="A94" s="6" t="inlineStr">
         <is>
-          <t>Imolote</t>
+          <t>Hines Portugal</t>
         </is>
       </c>
       <c r="B94" s="7" t="inlineStr">
@@ -4627,7 +4635,7 @@
       <c r="C94" s="8" t="inlineStr"/>
       <c r="D94" s="6" t="inlineStr">
         <is>
-          <t>Paulo Vaz Ferreira (sócio e CEO desde 2019, confiança moderada)</t>
+          <t>Vanessa Gelado (Senior Managing Director, Head of Southern Europe)</t>
         </is>
       </c>
       <c r="E94" s="6" t="inlineStr"/>
@@ -4635,24 +4643,24 @@
       <c r="G94" s="6" t="inlineStr"/>
       <c r="H94" s="6" t="inlineStr">
         <is>
-          <t>imolote.pt</t>
+          <t>hines.com</t>
         </is>
       </c>
       <c r="I94" s="8" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="J94" s="8" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Lisboa</t>
         </is>
       </c>
     </row>
     <row r="95" ht="26" customHeight="1">
       <c r="A95" s="6" t="inlineStr">
         <is>
-          <t>João Magalhães &amp; Alexandre Magalhães (promotores individuais)</t>
+          <t>Imolote</t>
         </is>
       </c>
       <c r="B95" s="7" t="inlineStr">
@@ -4663,13 +4671,17 @@
       <c r="C95" s="8" t="inlineStr"/>
       <c r="D95" s="6" t="inlineStr">
         <is>
-          <t>João Magalhães e Alexandre Magalhães (promotores individuais)</t>
+          <t>Paulo Vaz Ferreira (sócio e CEO desde 2019, confiança moderada)</t>
         </is>
       </c>
       <c r="E95" s="6" t="inlineStr"/>
       <c r="F95" s="6" t="inlineStr"/>
       <c r="G95" s="6" t="inlineStr"/>
-      <c r="H95" s="6" t="inlineStr"/>
+      <c r="H95" s="6" t="inlineStr">
+        <is>
+          <t>imolote.pt</t>
+        </is>
+      </c>
       <c r="I95" s="8" t="inlineStr">
         <is>
           <t>Porto</t>
@@ -4684,7 +4696,7 @@
     <row r="96" ht="26" customHeight="1">
       <c r="A96" s="6" t="inlineStr">
         <is>
-          <t>KKR Imo, S.A.</t>
+          <t>João Magalhães &amp; Alexandre Magalhães (promotores individuais)</t>
         </is>
       </c>
       <c r="B96" s="7" t="inlineStr">
@@ -4695,7 +4707,7 @@
       <c r="C96" s="8" t="inlineStr"/>
       <c r="D96" s="6" t="inlineStr">
         <is>
-          <t>Vera Kendall (administradora, dados de 2018 · confiança baixa)</t>
+          <t>João Magalhães e Alexandre Magalhães (promotores individuais)</t>
         </is>
       </c>
       <c r="E96" s="6" t="inlineStr"/>
@@ -4704,19 +4716,19 @@
       <c r="H96" s="6" t="inlineStr"/>
       <c r="I96" s="8" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Porto</t>
         </is>
       </c>
       <c r="J96" s="8" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Porto</t>
         </is>
       </c>
     </row>
     <row r="97" ht="26" customHeight="1">
       <c r="A97" s="6" t="inlineStr">
         <is>
-          <t>Neptune Developments</t>
+          <t>KKR Imo, S.A.</t>
         </is>
       </c>
       <c r="B97" s="7" t="inlineStr">
@@ -4725,18 +4737,18 @@
         </is>
       </c>
       <c r="C97" s="8" t="inlineStr"/>
-      <c r="D97" s="6" t="inlineStr"/>
+      <c r="D97" s="6" t="inlineStr">
+        <is>
+          <t>Vera Kendall (administradora, dados de 2018 · confiança baixa)</t>
+        </is>
+      </c>
       <c r="E97" s="6" t="inlineStr"/>
       <c r="F97" s="6" t="inlineStr"/>
       <c r="G97" s="6" t="inlineStr"/>
-      <c r="H97" s="6" t="inlineStr">
-        <is>
-          <t>neptune-developments.com</t>
-        </is>
-      </c>
+      <c r="H97" s="6" t="inlineStr"/>
       <c r="I97" s="8" t="inlineStr">
         <is>
-          <t>Cascais</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="J97" s="8" t="inlineStr">
@@ -4748,7 +4760,7 @@
     <row r="98" ht="26" customHeight="1">
       <c r="A98" s="6" t="inlineStr">
         <is>
-          <t>Onyria Group</t>
+          <t>Neptune Developments</t>
         </is>
       </c>
       <c r="B98" s="7" t="inlineStr">
@@ -4757,17 +4769,13 @@
         </is>
       </c>
       <c r="C98" s="8" t="inlineStr"/>
-      <c r="D98" s="6" t="inlineStr">
-        <is>
-          <t>José Carlos Pinto Coelho (fundador, 1986)</t>
-        </is>
-      </c>
+      <c r="D98" s="6" t="inlineStr"/>
       <c r="E98" s="6" t="inlineStr"/>
       <c r="F98" s="6" t="inlineStr"/>
       <c r="G98" s="6" t="inlineStr"/>
       <c r="H98" s="6" t="inlineStr">
         <is>
-          <t>onyriagroup.com</t>
+          <t>neptune-developments.com</t>
         </is>
       </c>
       <c r="I98" s="8" t="inlineStr">
@@ -4784,7 +4792,7 @@
     <row r="99" ht="26" customHeight="1">
       <c r="A99" s="6" t="inlineStr">
         <is>
-          <t>Portaviv</t>
+          <t>Onyria Group</t>
         </is>
       </c>
       <c r="B99" s="7" t="inlineStr">
@@ -4795,28 +4803,32 @@
       <c r="C99" s="8" t="inlineStr"/>
       <c r="D99" s="6" t="inlineStr">
         <is>
-          <t>Nuno Cunha (Managing Director)</t>
+          <t>José Carlos Pinto Coelho (fundador, 1986)</t>
         </is>
       </c>
       <c r="E99" s="6" t="inlineStr"/>
       <c r="F99" s="6" t="inlineStr"/>
       <c r="G99" s="6" t="inlineStr"/>
-      <c r="H99" s="6" t="inlineStr"/>
+      <c r="H99" s="6" t="inlineStr">
+        <is>
+          <t>onyriagroup.com</t>
+        </is>
+      </c>
       <c r="I99" s="8" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Cascais</t>
         </is>
       </c>
       <c r="J99" s="8" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Lisboa</t>
         </is>
       </c>
     </row>
     <row r="100" ht="26" customHeight="1">
       <c r="A100" s="6" t="inlineStr">
         <is>
-          <t>REABILITA</t>
+          <t>Portaviv</t>
         </is>
       </c>
       <c r="B100" s="7" t="inlineStr">
@@ -4825,30 +4837,30 @@
         </is>
       </c>
       <c r="C100" s="8" t="inlineStr"/>
-      <c r="D100" s="6" t="inlineStr"/>
+      <c r="D100" s="6" t="inlineStr">
+        <is>
+          <t>Nuno Cunha (Managing Director)</t>
+        </is>
+      </c>
       <c r="E100" s="6" t="inlineStr"/>
       <c r="F100" s="6" t="inlineStr"/>
       <c r="G100" s="6" t="inlineStr"/>
-      <c r="H100" s="6" t="inlineStr">
-        <is>
-          <t>reabilita.pt</t>
-        </is>
-      </c>
+      <c r="H100" s="6" t="inlineStr"/>
       <c r="I100" s="8" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Porto</t>
         </is>
       </c>
       <c r="J100" s="8" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Porto</t>
         </is>
       </c>
     </row>
     <row r="101" ht="26" customHeight="1">
       <c r="A101" s="6" t="inlineStr">
         <is>
-          <t>REDASSET</t>
+          <t>REABILITA</t>
         </is>
       </c>
       <c r="B101" s="7" t="inlineStr">
@@ -4861,10 +4873,14 @@
       <c r="E101" s="6" t="inlineStr"/>
       <c r="F101" s="6" t="inlineStr"/>
       <c r="G101" s="6" t="inlineStr"/>
-      <c r="H101" s="6" t="inlineStr"/>
+      <c r="H101" s="6" t="inlineStr">
+        <is>
+          <t>reabilita.pt</t>
+        </is>
+      </c>
       <c r="I101" s="8" t="inlineStr">
         <is>
-          <t>Amadora</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="J101" s="8" t="inlineStr">
@@ -4876,7 +4892,7 @@
     <row r="102" ht="26" customHeight="1">
       <c r="A102" s="6" t="inlineStr">
         <is>
-          <t>RM Promo (JV M2O Group / RJB Home)</t>
+          <t>REDASSET</t>
         </is>
       </c>
       <c r="B102" s="7" t="inlineStr">
@@ -4892,19 +4908,19 @@
       <c r="H102" s="6" t="inlineStr"/>
       <c r="I102" s="8" t="inlineStr">
         <is>
-          <t>Matosinhos</t>
+          <t>Amadora</t>
         </is>
       </c>
       <c r="J102" s="8" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Lisboa</t>
         </is>
       </c>
     </row>
     <row r="103" ht="26" customHeight="1">
       <c r="A103" s="6" t="inlineStr">
         <is>
-          <t>SGAL – Sociedade Gestora da Alta de Lisboa</t>
+          <t>RM Promo (JV M2O Group / RJB Home)</t>
         </is>
       </c>
       <c r="B103" s="7" t="inlineStr">
@@ -4917,26 +4933,22 @@
       <c r="E103" s="6" t="inlineStr"/>
       <c r="F103" s="6" t="inlineStr"/>
       <c r="G103" s="6" t="inlineStr"/>
-      <c r="H103" s="6" t="inlineStr">
-        <is>
-          <t>altadelisboa.com</t>
-        </is>
-      </c>
+      <c r="H103" s="6" t="inlineStr"/>
       <c r="I103" s="8" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Matosinhos</t>
         </is>
       </c>
       <c r="J103" s="8" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Porto</t>
         </is>
       </c>
     </row>
     <row r="104" ht="26" customHeight="1">
       <c r="A104" s="6" t="inlineStr">
         <is>
-          <t>Shalu Investments</t>
+          <t>Selicomi Portugal (Victoria Group)</t>
         </is>
       </c>
       <c r="B104" s="7" t="inlineStr">
@@ -4945,34 +4957,26 @@
         </is>
       </c>
       <c r="C104" s="8" t="inlineStr"/>
-      <c r="D104" s="6" t="inlineStr">
-        <is>
-          <t>Itai Fridman (Founder &amp; Managing Director)</t>
-        </is>
-      </c>
+      <c r="D104" s="6" t="inlineStr"/>
       <c r="E104" s="6" t="inlineStr"/>
       <c r="F104" s="6" t="inlineStr"/>
       <c r="G104" s="6" t="inlineStr"/>
-      <c r="H104" s="6" t="inlineStr">
-        <is>
-          <t>shaluinvest.pt</t>
-        </is>
-      </c>
+      <c r="H104" s="6" t="inlineStr"/>
       <c r="I104" s="8" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="J104" s="8" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Lisboa</t>
         </is>
       </c>
     </row>
     <row r="105" ht="26" customHeight="1">
       <c r="A105" s="6" t="inlineStr">
         <is>
-          <t>Taga Urbanic</t>
+          <t>SGAL – Sociedade Gestora da Alta de Lisboa</t>
         </is>
       </c>
       <c r="B105" s="7" t="inlineStr">
@@ -4985,130 +4989,122 @@
       <c r="E105" s="6" t="inlineStr"/>
       <c r="F105" s="6" t="inlineStr"/>
       <c r="G105" s="6" t="inlineStr"/>
-      <c r="H105" s="6" t="inlineStr"/>
+      <c r="H105" s="6" t="inlineStr">
+        <is>
+          <t>altadelisboa.com</t>
+        </is>
+      </c>
       <c r="I105" s="8" t="inlineStr">
         <is>
-          <t>Maia</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="J105" s="8" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Lisboa</t>
         </is>
       </c>
     </row>
     <row r="106" ht="26" customHeight="1">
       <c r="A106" s="6" t="inlineStr">
         <is>
-          <t>Amorim Luxury</t>
-        </is>
-      </c>
-      <c r="B106" s="8" t="inlineStr">
-        <is>
-          <t>Nao</t>
+          <t>Shalu Investments</t>
+        </is>
+      </c>
+      <c r="B106" s="7" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
       <c r="C106" s="8" t="inlineStr"/>
       <c r="D106" s="6" t="inlineStr">
         <is>
-          <t>Miguel Guedes de Sousa (Founder &amp; CEO)</t>
-        </is>
-      </c>
-      <c r="E106" s="9" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/miguelguedesdesousa/</t>
-        </is>
-      </c>
+          <t>Itai Fridman (Founder &amp; Managing Director)</t>
+        </is>
+      </c>
+      <c r="E106" s="6" t="inlineStr"/>
       <c r="F106" s="6" t="inlineStr"/>
       <c r="G106" s="6" t="inlineStr"/>
-      <c r="H106" s="6" t="inlineStr"/>
+      <c r="H106" s="6" t="inlineStr">
+        <is>
+          <t>shaluinvest.pt</t>
+        </is>
+      </c>
       <c r="I106" s="8" t="inlineStr">
         <is>
-          <t>Lisboa/Grândola/Lagoa</t>
+          <t>Porto</t>
         </is>
       </c>
       <c r="J106" s="8" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Porto</t>
         </is>
       </c>
     </row>
     <row r="107" ht="26" customHeight="1">
       <c r="A107" s="6" t="inlineStr">
         <is>
-          <t>Emblezart</t>
-        </is>
-      </c>
-      <c r="B107" s="8" t="inlineStr">
-        <is>
-          <t>Nao</t>
+          <t>Square Asset Management</t>
+        </is>
+      </c>
+      <c r="B107" s="7" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
       <c r="C107" s="8" t="inlineStr"/>
-      <c r="D107" s="6" t="inlineStr">
-        <is>
-          <t>David Faria (CEO e sócio único)</t>
-        </is>
-      </c>
-      <c r="E107" s="9" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/david-faria-a301a466/</t>
-        </is>
-      </c>
+      <c r="D107" s="6" t="inlineStr"/>
+      <c r="E107" s="6" t="inlineStr"/>
       <c r="F107" s="6" t="inlineStr"/>
       <c r="G107" s="6" t="inlineStr"/>
-      <c r="H107" s="6" t="inlineStr"/>
+      <c r="H107" s="6" t="inlineStr">
+        <is>
+          <t>squaream.pt</t>
+        </is>
+      </c>
       <c r="I107" s="8" t="inlineStr">
         <is>
-          <t>Guimarães</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="J107" s="8" t="inlineStr">
         <is>
-          <t>Braga</t>
+          <t>Lisboa</t>
         </is>
       </c>
     </row>
     <row r="108" ht="26" customHeight="1">
       <c r="A108" s="6" t="inlineStr">
         <is>
-          <t>Grupo Azinor</t>
-        </is>
-      </c>
-      <c r="B108" s="8" t="inlineStr">
-        <is>
-          <t>Nao</t>
+          <t>Taga Urbanic</t>
+        </is>
+      </c>
+      <c r="B108" s="7" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
       <c r="C108" s="8" t="inlineStr"/>
-      <c r="D108" s="6" t="inlineStr">
-        <is>
-          <t>Carlos Silva Neves (administrador)</t>
-        </is>
-      </c>
-      <c r="E108" s="9" t="inlineStr">
-        <is>
-          <t>https://pt.linkedin.com/in/carlos-silva-neves-3b0711142</t>
-        </is>
-      </c>
+      <c r="D108" s="6" t="inlineStr"/>
+      <c r="E108" s="6" t="inlineStr"/>
       <c r="F108" s="6" t="inlineStr"/>
       <c r="G108" s="6" t="inlineStr"/>
       <c r="H108" s="6" t="inlineStr"/>
       <c r="I108" s="8" t="inlineStr">
         <is>
-          <t>Oeiras</t>
+          <t>Maia</t>
         </is>
       </c>
       <c r="J108" s="8" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Porto</t>
         </is>
       </c>
     </row>
     <row r="109" ht="26" customHeight="1">
       <c r="A109" s="6" t="inlineStr">
         <is>
-          <t>JPAIVA Investimentos / JPAIVA Engenharia e Construção</t>
+          <t>Amorim Luxury</t>
         </is>
       </c>
       <c r="B109" s="8" t="inlineStr">
@@ -5119,36 +5115,32 @@
       <c r="C109" s="8" t="inlineStr"/>
       <c r="D109" s="6" t="inlineStr">
         <is>
-          <t>Igor Castro (CEO)</t>
+          <t>Miguel Guedes de Sousa (Founder &amp; CEO)</t>
         </is>
       </c>
       <c r="E109" s="9" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/igor-castro-a0026b22b/</t>
+          <t>https://www.linkedin.com/in/miguelguedesdesousa/</t>
         </is>
       </c>
       <c r="F109" s="6" t="inlineStr"/>
       <c r="G109" s="6" t="inlineStr"/>
-      <c r="H109" s="6" t="inlineStr">
-        <is>
-          <t>jpaiva.pt</t>
-        </is>
-      </c>
+      <c r="H109" s="6" t="inlineStr"/>
       <c r="I109" s="8" t="inlineStr">
         <is>
-          <t>Coimbra</t>
+          <t>Lisboa/Grândola/Lagoa</t>
         </is>
       </c>
       <c r="J109" s="8" t="inlineStr">
         <is>
-          <t>Coimbra</t>
+          <t>Lisboa</t>
         </is>
       </c>
     </row>
     <row r="110" ht="26" customHeight="1">
       <c r="A110" s="6" t="inlineStr">
         <is>
-          <t>Mello RDC</t>
+          <t>Emblezart</t>
         </is>
       </c>
       <c r="B110" s="8" t="inlineStr">
@@ -5159,36 +5151,32 @@
       <c r="C110" s="8" t="inlineStr"/>
       <c r="D110" s="6" t="inlineStr">
         <is>
-          <t>António Ribeiro da Cunha (CEO)</t>
+          <t>David Faria (CEO e sócio único)</t>
         </is>
       </c>
       <c r="E110" s="9" t="inlineStr">
         <is>
-          <t>https://pt.linkedin.com/in/ant%C3%B3nio-ribeiro-da-cunha-77b974112</t>
+          <t>https://www.linkedin.com/in/david-faria-a301a466/</t>
         </is>
       </c>
       <c r="F110" s="6" t="inlineStr"/>
       <c r="G110" s="6" t="inlineStr"/>
-      <c r="H110" s="6" t="inlineStr">
-        <is>
-          <t>mellordc.pt</t>
-        </is>
-      </c>
+      <c r="H110" s="6" t="inlineStr"/>
       <c r="I110" s="8" t="inlineStr">
         <is>
-          <t>Grândola (Melides)</t>
+          <t>Guimarães</t>
         </is>
       </c>
       <c r="J110" s="8" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Braga</t>
         </is>
       </c>
     </row>
     <row r="111" ht="26" customHeight="1">
       <c r="A111" s="6" t="inlineStr">
         <is>
-          <t>Ombria Resort (Grupo Pontos)</t>
+          <t>Grupo Azinor</t>
         </is>
       </c>
       <c r="B111" s="8" t="inlineStr">
@@ -5199,36 +5187,32 @@
       <c r="C111" s="8" t="inlineStr"/>
       <c r="D111" s="6" t="inlineStr">
         <is>
-          <t>Patrick Freeman (CEO Ombria desde 2023)· CEO do Grupo Pontos é Timo Kokkila</t>
+          <t>Carlos Silva Neves (administrador)</t>
         </is>
       </c>
       <c r="E111" s="9" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/patricksfreeman/</t>
+          <t>https://pt.linkedin.com/in/carlos-silva-neves-3b0711142</t>
         </is>
       </c>
       <c r="F111" s="6" t="inlineStr"/>
       <c r="G111" s="6" t="inlineStr"/>
-      <c r="H111" s="6" t="inlineStr">
-        <is>
-          <t>ombria.com</t>
-        </is>
-      </c>
+      <c r="H111" s="6" t="inlineStr"/>
       <c r="I111" s="8" t="inlineStr">
         <is>
-          <t>Loulé</t>
+          <t>Oeiras</t>
         </is>
       </c>
       <c r="J111" s="8" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Lisboa</t>
         </is>
       </c>
     </row>
     <row r="112" ht="26" customHeight="1">
       <c r="A112" s="6" t="inlineStr">
         <is>
-          <t>Soccal &amp; Vaz Invest</t>
+          <t>JPAIVA Investimentos / JPAIVA Engenharia e Construção</t>
         </is>
       </c>
       <c r="B112" s="8" t="inlineStr">
@@ -5239,36 +5223,36 @@
       <c r="C112" s="8" t="inlineStr"/>
       <c r="D112" s="6" t="inlineStr">
         <is>
-          <t>António Vaz (fundador e CEO)</t>
+          <t>Igor Castro (CEO)</t>
         </is>
       </c>
       <c r="E112" s="9" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/antonio-vaz-9444998a/</t>
+          <t>https://www.linkedin.com/in/igor-castro-a0026b22b/</t>
         </is>
       </c>
       <c r="F112" s="6" t="inlineStr"/>
       <c r="G112" s="6" t="inlineStr"/>
       <c r="H112" s="6" t="inlineStr">
         <is>
-          <t>soccal-vaz.com</t>
+          <t>jpaiva.pt</t>
         </is>
       </c>
       <c r="I112" s="8" t="inlineStr">
         <is>
-          <t>Sines</t>
+          <t>Coimbra</t>
         </is>
       </c>
       <c r="J112" s="8" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Coimbra</t>
         </is>
       </c>
     </row>
     <row r="113" ht="26" customHeight="1">
       <c r="A113" s="6" t="inlineStr">
         <is>
-          <t>Solid Sentinel</t>
+          <t>Mello RDC</t>
         </is>
       </c>
       <c r="B113" s="8" t="inlineStr">
@@ -5279,24 +5263,24 @@
       <c r="C113" s="8" t="inlineStr"/>
       <c r="D113" s="6" t="inlineStr">
         <is>
-          <t>Alain Gross (Co-Founder e CEO)</t>
+          <t>António Ribeiro da Cunha (CEO)</t>
         </is>
       </c>
       <c r="E113" s="9" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/alain-gross-3351411/</t>
+          <t>https://pt.linkedin.com/in/ant%C3%B3nio-ribeiro-da-cunha-77b974112</t>
         </is>
       </c>
       <c r="F113" s="6" t="inlineStr"/>
       <c r="G113" s="6" t="inlineStr"/>
       <c r="H113" s="6" t="inlineStr">
         <is>
-          <t>solidsentinel.pt</t>
+          <t>mellordc.pt</t>
         </is>
       </c>
       <c r="I113" s="8" t="inlineStr">
         <is>
-          <t>Barreiro</t>
+          <t>Grândola (Melides)</t>
         </is>
       </c>
       <c r="J113" s="8" t="inlineStr">
@@ -5308,7 +5292,7 @@
     <row r="114" ht="26" customHeight="1">
       <c r="A114" s="6" t="inlineStr">
         <is>
-          <t>Sonae Sierra</t>
+          <t>Ombria Resort (Grupo Pontos)</t>
         </is>
       </c>
       <c r="B114" s="8" t="inlineStr">
@@ -5319,36 +5303,36 @@
       <c r="C114" s="8" t="inlineStr"/>
       <c r="D114" s="6" t="inlineStr">
         <is>
-          <t>Fernando Guedes de Oliveira (CEO)</t>
+          <t>Patrick Freeman (CEO Ombria desde 2023)· CEO do Grupo Pontos é Timo Kokkila</t>
         </is>
       </c>
       <c r="E114" s="9" t="inlineStr">
         <is>
-          <t>https://pt.linkedin.com/in/fernando-oliveira-9622b817</t>
+          <t>https://www.linkedin.com/in/patricksfreeman/</t>
         </is>
       </c>
       <c r="F114" s="6" t="inlineStr"/>
       <c r="G114" s="6" t="inlineStr"/>
       <c r="H114" s="6" t="inlineStr">
         <is>
-          <t>sonaesierra.com</t>
+          <t>ombria.com</t>
         </is>
       </c>
       <c r="I114" s="8" t="inlineStr">
         <is>
-          <t>Lisboa/Porto</t>
+          <t>Loulé</t>
         </is>
       </c>
       <c r="J114" s="8" t="inlineStr">
         <is>
-          <t>nacional</t>
+          <t>Faro</t>
         </is>
       </c>
     </row>
     <row r="115" ht="26" customHeight="1">
       <c r="A115" s="6" t="inlineStr">
         <is>
-          <t>Square View</t>
+          <t>Soccal &amp; Vaz Invest</t>
         </is>
       </c>
       <c r="B115" s="8" t="inlineStr">
@@ -5359,36 +5343,36 @@
       <c r="C115" s="8" t="inlineStr"/>
       <c r="D115" s="6" t="inlineStr">
         <is>
-          <t>Luis Horta e Costa (CEO/Fundador)</t>
+          <t>António Vaz (fundador e CEO)</t>
         </is>
       </c>
       <c r="E115" s="9" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/luis-horta-e-costa-377552241/</t>
+          <t>https://www.linkedin.com/in/antonio-vaz-9444998a/</t>
         </is>
       </c>
       <c r="F115" s="6" t="inlineStr"/>
       <c r="G115" s="6" t="inlineStr"/>
       <c r="H115" s="6" t="inlineStr">
         <is>
-          <t>squareview.pt</t>
+          <t>soccal-vaz.com</t>
         </is>
       </c>
       <c r="I115" s="8" t="inlineStr">
         <is>
-          <t>Lisboa/Ericeira/Melides</t>
+          <t>Sines</t>
         </is>
       </c>
       <c r="J115" s="8" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Setúbal</t>
         </is>
       </c>
     </row>
     <row r="116" ht="26" customHeight="1">
       <c r="A116" s="6" t="inlineStr">
         <is>
-          <t>Algarve Property Shops</t>
+          <t>Solid Sentinel</t>
         </is>
       </c>
       <c r="B116" s="8" t="inlineStr">
@@ -5397,26 +5381,38 @@
         </is>
       </c>
       <c r="C116" s="8" t="inlineStr"/>
-      <c r="D116" s="6" t="inlineStr"/>
-      <c r="E116" s="6" t="inlineStr"/>
+      <c r="D116" s="6" t="inlineStr">
+        <is>
+          <t>Alain Gross (Co-Founder e CEO)</t>
+        </is>
+      </c>
+      <c r="E116" s="9" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/alain-gross-3351411/</t>
+        </is>
+      </c>
       <c r="F116" s="6" t="inlineStr"/>
       <c r="G116" s="6" t="inlineStr"/>
-      <c r="H116" s="6" t="inlineStr"/>
+      <c r="H116" s="6" t="inlineStr">
+        <is>
+          <t>solidsentinel.pt</t>
+        </is>
+      </c>
       <c r="I116" s="8" t="inlineStr">
         <is>
-          <t>Tavira</t>
+          <t>Barreiro</t>
         </is>
       </c>
       <c r="J116" s="8" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Setúbal</t>
         </is>
       </c>
     </row>
     <row r="117" ht="26" customHeight="1">
       <c r="A117" s="6" t="inlineStr">
         <is>
-          <t>Aresta Vitalicia</t>
+          <t>Sonae Sierra</t>
         </is>
       </c>
       <c r="B117" s="8" t="inlineStr">
@@ -5425,26 +5421,38 @@
         </is>
       </c>
       <c r="C117" s="8" t="inlineStr"/>
-      <c r="D117" s="6" t="inlineStr"/>
-      <c r="E117" s="6" t="inlineStr"/>
+      <c r="D117" s="6" t="inlineStr">
+        <is>
+          <t>Fernando Guedes de Oliveira (CEO)</t>
+        </is>
+      </c>
+      <c r="E117" s="9" t="inlineStr">
+        <is>
+          <t>https://pt.linkedin.com/in/fernando-oliveira-9622b817</t>
+        </is>
+      </c>
       <c r="F117" s="6" t="inlineStr"/>
       <c r="G117" s="6" t="inlineStr"/>
-      <c r="H117" s="6" t="inlineStr"/>
+      <c r="H117" s="6" t="inlineStr">
+        <is>
+          <t>sonaesierra.com</t>
+        </is>
+      </c>
       <c r="I117" s="8" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Lisboa/Porto</t>
         </is>
       </c>
       <c r="J117" s="8" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>nacional</t>
         </is>
       </c>
     </row>
     <row r="118" ht="26" customHeight="1">
       <c r="A118" s="6" t="inlineStr">
         <is>
-          <t>Arrow Global Portugal</t>
+          <t>Square View</t>
         </is>
       </c>
       <c r="B118" s="8" t="inlineStr">
@@ -5455,28 +5463,36 @@
       <c r="C118" s="8" t="inlineStr"/>
       <c r="D118" s="6" t="inlineStr">
         <is>
-          <t>João Bugalho (CEO)</t>
-        </is>
-      </c>
-      <c r="E118" s="6" t="inlineStr"/>
+          <t>Luis Horta e Costa (CEO/Fundador)</t>
+        </is>
+      </c>
+      <c r="E118" s="9" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/luis-horta-e-costa-377552241/</t>
+        </is>
+      </c>
       <c r="F118" s="6" t="inlineStr"/>
       <c r="G118" s="6" t="inlineStr"/>
-      <c r="H118" s="6" t="inlineStr"/>
+      <c r="H118" s="6" t="inlineStr">
+        <is>
+          <t>squareview.pt</t>
+        </is>
+      </c>
       <c r="I118" s="8" t="inlineStr">
         <is>
-          <t>Loulé (Almancil/Quinta do Lago)</t>
+          <t>Lisboa/Ericeira/Melides</t>
         </is>
       </c>
       <c r="J118" s="8" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Lisboa</t>
         </is>
       </c>
     </row>
     <row r="119" ht="26" customHeight="1">
       <c r="A119" s="6" t="inlineStr">
         <is>
-          <t>Baltor – Engenharia e Construção</t>
+          <t>Algarve Property Shops</t>
         </is>
       </c>
       <c r="B119" s="8" t="inlineStr">
@@ -5485,34 +5501,26 @@
         </is>
       </c>
       <c r="C119" s="8" t="inlineStr"/>
-      <c r="D119" s="6" t="inlineStr">
-        <is>
-          <t>Paulo Balinha e Bruno Torres (fundadores, 2008)</t>
-        </is>
-      </c>
+      <c r="D119" s="6" t="inlineStr"/>
       <c r="E119" s="6" t="inlineStr"/>
       <c r="F119" s="6" t="inlineStr"/>
       <c r="G119" s="6" t="inlineStr"/>
-      <c r="H119" s="6" t="inlineStr">
-        <is>
-          <t>baltor.pt</t>
-        </is>
-      </c>
+      <c r="H119" s="6" t="inlineStr"/>
       <c r="I119" s="8" t="inlineStr">
         <is>
-          <t>Setúbal (sede Viana do Castelo)</t>
+          <t>Tavira</t>
         </is>
       </c>
       <c r="J119" s="8" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Faro</t>
         </is>
       </c>
     </row>
     <row r="120" ht="26" customHeight="1">
       <c r="A120" s="6" t="inlineStr">
         <is>
-          <t>Bond Group</t>
+          <t>Aresta Vitalicia</t>
         </is>
       </c>
       <c r="B120" s="8" t="inlineStr">
@@ -5528,19 +5536,19 @@
       <c r="H120" s="6" t="inlineStr"/>
       <c r="I120" s="8" t="inlineStr">
         <is>
-          <t>Amares</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="J120" s="8" t="inlineStr">
         <is>
-          <t>Braga</t>
+          <t>Setúbal</t>
         </is>
       </c>
     </row>
     <row r="121" ht="26" customHeight="1">
       <c r="A121" s="6" t="inlineStr">
         <is>
-          <t>Branco Real Estate</t>
+          <t>Arrow Global Portugal</t>
         </is>
       </c>
       <c r="B121" s="8" t="inlineStr">
@@ -5549,14 +5557,18 @@
         </is>
       </c>
       <c r="C121" s="8" t="inlineStr"/>
-      <c r="D121" s="6" t="inlineStr"/>
+      <c r="D121" s="6" t="inlineStr">
+        <is>
+          <t>João Bugalho (CEO)</t>
+        </is>
+      </c>
       <c r="E121" s="6" t="inlineStr"/>
       <c r="F121" s="6" t="inlineStr"/>
       <c r="G121" s="6" t="inlineStr"/>
       <c r="H121" s="6" t="inlineStr"/>
       <c r="I121" s="8" t="inlineStr">
         <is>
-          <t>Lagos</t>
+          <t>Loulé (Almancil/Quinta do Lago)</t>
         </is>
       </c>
       <c r="J121" s="8" t="inlineStr">
@@ -5568,7 +5580,7 @@
     <row r="122" ht="26" customHeight="1">
       <c r="A122" s="6" t="inlineStr">
         <is>
-          <t>Casas do Sotavento</t>
+          <t>Baltor – Engenharia e Construção</t>
         </is>
       </c>
       <c r="B122" s="8" t="inlineStr">
@@ -5577,30 +5589,34 @@
         </is>
       </c>
       <c r="C122" s="8" t="inlineStr"/>
-      <c r="D122" s="6" t="inlineStr"/>
+      <c r="D122" s="6" t="inlineStr">
+        <is>
+          <t>Paulo Balinha e Bruno Torres (fundadores, 2008)</t>
+        </is>
+      </c>
       <c r="E122" s="6" t="inlineStr"/>
       <c r="F122" s="6" t="inlineStr"/>
       <c r="G122" s="6" t="inlineStr"/>
       <c r="H122" s="6" t="inlineStr">
         <is>
-          <t>casasdosotavento.pt</t>
+          <t>baltor.pt</t>
         </is>
       </c>
       <c r="I122" s="8" t="inlineStr">
         <is>
-          <t>Tavira</t>
+          <t>Setúbal (sede Viana do Castelo)</t>
         </is>
       </c>
       <c r="J122" s="8" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Setúbal</t>
         </is>
       </c>
     </row>
     <row r="123" ht="26" customHeight="1">
       <c r="A123" s="6" t="inlineStr">
         <is>
-          <t>Confidential Sphere – Investimento Imobiliário</t>
+          <t>Bond Group</t>
         </is>
       </c>
       <c r="B123" s="8" t="inlineStr">
@@ -5616,19 +5632,19 @@
       <c r="H123" s="6" t="inlineStr"/>
       <c r="I123" s="8" t="inlineStr">
         <is>
-          <t>Silves</t>
+          <t>Amares</t>
         </is>
       </c>
       <c r="J123" s="8" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Braga</t>
         </is>
       </c>
     </row>
     <row r="124" ht="26" customHeight="1">
       <c r="A124" s="6" t="inlineStr">
         <is>
-          <t>CS Ribeiro</t>
+          <t>Branco Real Estate</t>
         </is>
       </c>
       <c r="B124" s="8" t="inlineStr">
@@ -5644,19 +5660,19 @@
       <c r="H124" s="6" t="inlineStr"/>
       <c r="I124" s="8" t="inlineStr">
         <is>
-          <t>Guarda (atua Viseu/Coimbra)</t>
+          <t>Lagos</t>
         </is>
       </c>
       <c r="J124" s="8" t="inlineStr">
         <is>
-          <t>Guarda</t>
+          <t>Faro</t>
         </is>
       </c>
     </row>
     <row r="125" ht="26" customHeight="1">
       <c r="A125" s="6" t="inlineStr">
         <is>
-          <t>Discovery Land Company</t>
+          <t>Casas do Sotavento</t>
         </is>
       </c>
       <c r="B125" s="8" t="inlineStr">
@@ -5671,24 +5687,24 @@
       <c r="G125" s="6" t="inlineStr"/>
       <c r="H125" s="6" t="inlineStr">
         <is>
-          <t>discoverylandco.com</t>
+          <t>casasdosotavento.pt</t>
         </is>
       </c>
       <c r="I125" s="8" t="inlineStr">
         <is>
-          <t>Grândola (Melides)</t>
+          <t>Tavira</t>
         </is>
       </c>
       <c r="J125" s="8" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Faro</t>
         </is>
       </c>
     </row>
     <row r="126" ht="26" customHeight="1">
       <c r="A126" s="6" t="inlineStr">
         <is>
-          <t>DUJA – Sociedade de Construções, Lda</t>
+          <t>Confidential Sphere – Investimento Imobiliário</t>
         </is>
       </c>
       <c r="B126" s="8" t="inlineStr">
@@ -5704,7 +5720,7 @@
       <c r="H126" s="6" t="inlineStr"/>
       <c r="I126" s="8" t="inlineStr">
         <is>
-          <t>Tavira</t>
+          <t>Silves</t>
         </is>
       </c>
       <c r="J126" s="8" t="inlineStr">
@@ -5716,7 +5732,7 @@
     <row r="127" ht="26" customHeight="1">
       <c r="A127" s="6" t="inlineStr">
         <is>
-          <t>Encobarra</t>
+          <t>CS Ribeiro</t>
         </is>
       </c>
       <c r="B127" s="8" t="inlineStr">
@@ -5725,30 +5741,26 @@
         </is>
       </c>
       <c r="C127" s="8" t="inlineStr"/>
-      <c r="D127" s="6" t="inlineStr">
-        <is>
-          <t>Aristides Alferes (administrador)</t>
-        </is>
-      </c>
+      <c r="D127" s="6" t="inlineStr"/>
       <c r="E127" s="6" t="inlineStr"/>
       <c r="F127" s="6" t="inlineStr"/>
       <c r="G127" s="6" t="inlineStr"/>
       <c r="H127" s="6" t="inlineStr"/>
       <c r="I127" s="8" t="inlineStr">
         <is>
-          <t>Aveiro (Aradas)</t>
+          <t>Guarda (atua Viseu/Coimbra)</t>
         </is>
       </c>
       <c r="J127" s="8" t="inlineStr">
         <is>
-          <t>Aveiro</t>
+          <t>Guarda</t>
         </is>
       </c>
     </row>
     <row r="128" ht="26" customHeight="1">
       <c r="A128" s="6" t="inlineStr">
         <is>
-          <t>Estrutural Group</t>
+          <t>Discovery Land Company</t>
         </is>
       </c>
       <c r="B128" s="8" t="inlineStr">
@@ -5757,30 +5769,30 @@
         </is>
       </c>
       <c r="C128" s="8" t="inlineStr"/>
-      <c r="D128" s="6" t="inlineStr">
-        <is>
-          <t>Hugo Mendes Pinto (Managing Partner)</t>
-        </is>
-      </c>
+      <c r="D128" s="6" t="inlineStr"/>
       <c r="E128" s="6" t="inlineStr"/>
       <c r="F128" s="6" t="inlineStr"/>
       <c r="G128" s="6" t="inlineStr"/>
-      <c r="H128" s="6" t="inlineStr"/>
+      <c r="H128" s="6" t="inlineStr">
+        <is>
+          <t>discoverylandco.com</t>
+        </is>
+      </c>
       <c r="I128" s="8" t="inlineStr">
         <is>
-          <t>Vila Franca de Xira</t>
+          <t>Grândola (Melides)</t>
         </is>
       </c>
       <c r="J128" s="8" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Setúbal</t>
         </is>
       </c>
     </row>
     <row r="129" ht="26" customHeight="1">
       <c r="A129" s="6" t="inlineStr">
         <is>
-          <t>Explorer Investments (Explorer Real Estate)</t>
+          <t>DUJA – Sociedade de Construções, Lda</t>
         </is>
       </c>
       <c r="B129" s="8" t="inlineStr">
@@ -5789,34 +5801,26 @@
         </is>
       </c>
       <c r="C129" s="8" t="inlineStr"/>
-      <c r="D129" s="6" t="inlineStr">
-        <is>
-          <t>Elizabeth Rothfield (CEO, Founding Partner)</t>
-        </is>
-      </c>
+      <c r="D129" s="6" t="inlineStr"/>
       <c r="E129" s="6" t="inlineStr"/>
       <c r="F129" s="6" t="inlineStr"/>
       <c r="G129" s="6" t="inlineStr"/>
-      <c r="H129" s="6" t="inlineStr">
-        <is>
-          <t>explorerinvestments.com</t>
-        </is>
-      </c>
+      <c r="H129" s="6" t="inlineStr"/>
       <c r="I129" s="8" t="inlineStr">
         <is>
-          <t>Sintra</t>
+          <t>Tavira</t>
         </is>
       </c>
       <c r="J129" s="8" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Faro</t>
         </is>
       </c>
     </row>
     <row r="130" ht="26" customHeight="1">
       <c r="A130" s="6" t="inlineStr">
         <is>
-          <t>Finangeste, S.A.</t>
+          <t>Encobarra</t>
         </is>
       </c>
       <c r="B130" s="8" t="inlineStr">
@@ -5827,7 +5831,7 @@
       <c r="C130" s="8" t="inlineStr"/>
       <c r="D130" s="6" t="inlineStr">
         <is>
-          <t>Paul Henri Schelfhout (Presidente do CA) / Armando Lacerda Queiroz (administrador)</t>
+          <t>Aristides Alferes (administrador)</t>
         </is>
       </c>
       <c r="E130" s="6" t="inlineStr"/>
@@ -5836,19 +5840,19 @@
       <c r="H130" s="6" t="inlineStr"/>
       <c r="I130" s="8" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Aveiro (Aradas)</t>
         </is>
       </c>
       <c r="J130" s="8" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Aveiro</t>
         </is>
       </c>
     </row>
     <row r="131" ht="26" customHeight="1">
       <c r="A131" s="6" t="inlineStr">
         <is>
-          <t>FourPromo, Lda (Grupo M2O)</t>
+          <t>Estrutural Group</t>
         </is>
       </c>
       <c r="B131" s="8" t="inlineStr">
@@ -5857,26 +5861,30 @@
         </is>
       </c>
       <c r="C131" s="8" t="inlineStr"/>
-      <c r="D131" s="6" t="inlineStr"/>
+      <c r="D131" s="6" t="inlineStr">
+        <is>
+          <t>Hugo Mendes Pinto (Managing Partner)</t>
+        </is>
+      </c>
       <c r="E131" s="6" t="inlineStr"/>
       <c r="F131" s="6" t="inlineStr"/>
       <c r="G131" s="6" t="inlineStr"/>
       <c r="H131" s="6" t="inlineStr"/>
       <c r="I131" s="8" t="inlineStr">
         <is>
-          <t>Loulé (Vilamoura)</t>
+          <t>Vila Franca de Xira</t>
         </is>
       </c>
       <c r="J131" s="8" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Lisboa</t>
         </is>
       </c>
     </row>
     <row r="132" ht="26" customHeight="1">
       <c r="A132" s="6" t="inlineStr">
         <is>
-          <t>Foz Gala Investments</t>
+          <t>Explorer Investments (Explorer Real Estate)</t>
         </is>
       </c>
       <c r="B132" s="8" t="inlineStr">
@@ -5885,26 +5893,34 @@
         </is>
       </c>
       <c r="C132" s="8" t="inlineStr"/>
-      <c r="D132" s="6" t="inlineStr"/>
+      <c r="D132" s="6" t="inlineStr">
+        <is>
+          <t>Elizabeth Rothfield (CEO, Founding Partner)</t>
+        </is>
+      </c>
       <c r="E132" s="6" t="inlineStr"/>
       <c r="F132" s="6" t="inlineStr"/>
       <c r="G132" s="6" t="inlineStr"/>
-      <c r="H132" s="6" t="inlineStr"/>
+      <c r="H132" s="6" t="inlineStr">
+        <is>
+          <t>explorerinvestments.com</t>
+        </is>
+      </c>
       <c r="I132" s="8" t="inlineStr">
         <is>
-          <t>Figueira da Foz</t>
+          <t>Sintra</t>
         </is>
       </c>
       <c r="J132" s="8" t="inlineStr">
         <is>
-          <t>Coimbra</t>
+          <t>Lisboa</t>
         </is>
       </c>
     </row>
     <row r="133" ht="26" customHeight="1">
       <c r="A133" s="6" t="inlineStr">
         <is>
-          <t>Galvana Investimentos Imobiliários e Turísticos, Lda</t>
+          <t>Finangeste, S.A.</t>
         </is>
       </c>
       <c r="B133" s="8" t="inlineStr">
@@ -5913,14 +5929,18 @@
         </is>
       </c>
       <c r="C133" s="8" t="inlineStr"/>
-      <c r="D133" s="6" t="inlineStr"/>
+      <c r="D133" s="6" t="inlineStr">
+        <is>
+          <t>Paul Henri Schelfhout (Presidente do CA) / Armando Lacerda Queiroz (administrador)</t>
+        </is>
+      </c>
       <c r="E133" s="6" t="inlineStr"/>
       <c r="F133" s="6" t="inlineStr"/>
       <c r="G133" s="6" t="inlineStr"/>
       <c r="H133" s="6" t="inlineStr"/>
       <c r="I133" s="8" t="inlineStr">
         <is>
-          <t>Albufeira</t>
+          <t>Faro</t>
         </is>
       </c>
       <c r="J133" s="8" t="inlineStr">
@@ -5932,7 +5952,7 @@
     <row r="134" ht="26" customHeight="1">
       <c r="A134" s="6" t="inlineStr">
         <is>
-          <t>Genuino Investments</t>
+          <t>FourPromo, Lda (Grupo M2O)</t>
         </is>
       </c>
       <c r="B134" s="8" t="inlineStr">
@@ -5945,14 +5965,10 @@
       <c r="E134" s="6" t="inlineStr"/>
       <c r="F134" s="6" t="inlineStr"/>
       <c r="G134" s="6" t="inlineStr"/>
-      <c r="H134" s="6" t="inlineStr">
-        <is>
-          <t>genuinoinvestments.com</t>
-        </is>
-      </c>
+      <c r="H134" s="6" t="inlineStr"/>
       <c r="I134" s="8" t="inlineStr">
         <is>
-          <t>Portimão</t>
+          <t>Loulé (Vilamoura)</t>
         </is>
       </c>
       <c r="J134" s="8" t="inlineStr">
@@ -5964,7 +5980,7 @@
     <row r="135" ht="26" customHeight="1">
       <c r="A135" s="6" t="inlineStr">
         <is>
-          <t>GFH (Grupo Ferreira Holding) / Ferreira Build Power (marca BeLiving)</t>
+          <t>Foz Gala Investments</t>
         </is>
       </c>
       <c r="B135" s="8" t="inlineStr">
@@ -5973,34 +5989,26 @@
         </is>
       </c>
       <c r="C135" s="8" t="inlineStr"/>
-      <c r="D135" s="6" t="inlineStr">
-        <is>
-          <t>Joaquim Silva (CEO Ferreira Build Power)</t>
-        </is>
-      </c>
+      <c r="D135" s="6" t="inlineStr"/>
       <c r="E135" s="6" t="inlineStr"/>
       <c r="F135" s="6" t="inlineStr"/>
       <c r="G135" s="6" t="inlineStr"/>
-      <c r="H135" s="6" t="inlineStr">
-        <is>
-          <t>ferreirabuildpower.com</t>
-        </is>
-      </c>
+      <c r="H135" s="6" t="inlineStr"/>
       <c r="I135" s="8" t="inlineStr">
         <is>
-          <t>Faro/Loulé</t>
+          <t>Figueira da Foz</t>
         </is>
       </c>
       <c r="J135" s="8" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Coimbra</t>
         </is>
       </c>
     </row>
     <row r="136" ht="26" customHeight="1">
       <c r="A136" s="6" t="inlineStr">
         <is>
-          <t>Glowing</t>
+          <t>Galvana Investimentos Imobiliários e Turísticos, Lda</t>
         </is>
       </c>
       <c r="B136" s="8" t="inlineStr">
@@ -6013,26 +6021,22 @@
       <c r="E136" s="6" t="inlineStr"/>
       <c r="F136" s="6" t="inlineStr"/>
       <c r="G136" s="6" t="inlineStr"/>
-      <c r="H136" s="6" t="inlineStr">
-        <is>
-          <t>glowing.pt</t>
-        </is>
-      </c>
+      <c r="H136" s="6" t="inlineStr"/>
       <c r="I136" s="8" t="inlineStr">
         <is>
-          <t>Alcácer do Sal</t>
+          <t>Albufeira</t>
         </is>
       </c>
       <c r="J136" s="8" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Faro</t>
         </is>
       </c>
     </row>
     <row r="137" ht="26" customHeight="1">
       <c r="A137" s="6" t="inlineStr">
         <is>
-          <t>Grupo A. Silva &amp; Silva</t>
+          <t>Genuino Investments</t>
         </is>
       </c>
       <c r="B137" s="8" t="inlineStr">
@@ -6045,22 +6049,26 @@
       <c r="E137" s="6" t="inlineStr"/>
       <c r="F137" s="6" t="inlineStr"/>
       <c r="G137" s="6" t="inlineStr"/>
-      <c r="H137" s="6" t="inlineStr"/>
+      <c r="H137" s="6" t="inlineStr">
+        <is>
+          <t>genuinoinvestments.com</t>
+        </is>
+      </c>
       <c r="I137" s="8" t="inlineStr">
         <is>
-          <t>Seixal</t>
+          <t>Portimão</t>
         </is>
       </c>
       <c r="J137" s="8" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Faro</t>
         </is>
       </c>
     </row>
     <row r="138" ht="26" customHeight="1">
       <c r="A138" s="6" t="inlineStr">
         <is>
-          <t>Grupo André Guimarães (Portugal)</t>
+          <t>GFH (Grupo Ferreira Holding) / Ferreira Build Power (marca BeLiving)</t>
         </is>
       </c>
       <c r="B138" s="8" t="inlineStr">
@@ -6071,7 +6079,7 @@
       <c r="C138" s="8" t="inlineStr"/>
       <c r="D138" s="6" t="inlineStr">
         <is>
-          <t>Fundador falecido· hoje liderado pelos filhos (Brasil), sem responsável PT confirmado</t>
+          <t>Joaquim Silva (CEO Ferreira Build Power)</t>
         </is>
       </c>
       <c r="E138" s="6" t="inlineStr"/>
@@ -6079,16 +6087,24 @@
       <c r="G138" s="6" t="inlineStr"/>
       <c r="H138" s="6" t="inlineStr">
         <is>
-          <t>andreguimaraes.com.br</t>
-        </is>
-      </c>
-      <c r="I138" s="8" t="inlineStr"/>
-      <c r="J138" s="8" t="inlineStr"/>
+          <t>ferreirabuildpower.com</t>
+        </is>
+      </c>
+      <c r="I138" s="8" t="inlineStr">
+        <is>
+          <t>Faro/Loulé</t>
+        </is>
+      </c>
+      <c r="J138" s="8" t="inlineStr">
+        <is>
+          <t>Faro</t>
+        </is>
+      </c>
     </row>
     <row r="139" ht="26" customHeight="1">
       <c r="A139" s="6" t="inlineStr">
         <is>
-          <t>Grupo André Jordan</t>
+          <t>Glowing</t>
         </is>
       </c>
       <c r="B139" s="8" t="inlineStr">
@@ -6097,34 +6113,30 @@
         </is>
       </c>
       <c r="C139" s="8" t="inlineStr"/>
-      <c r="D139" s="6" t="inlineStr">
-        <is>
-          <t>Gilberto Jordan (CEO desde 2009 · sucede a André Jordan, falecido 2024)</t>
-        </is>
-      </c>
+      <c r="D139" s="6" t="inlineStr"/>
       <c r="E139" s="6" t="inlineStr"/>
       <c r="F139" s="6" t="inlineStr"/>
       <c r="G139" s="6" t="inlineStr"/>
       <c r="H139" s="6" t="inlineStr">
         <is>
-          <t>andrejordangroup.pt</t>
+          <t>glowing.pt</t>
         </is>
       </c>
       <c r="I139" s="8" t="inlineStr">
         <is>
-          <t>Sintra</t>
+          <t>Alcácer do Sal</t>
         </is>
       </c>
       <c r="J139" s="8" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Setúbal</t>
         </is>
       </c>
     </row>
     <row r="140" ht="26" customHeight="1">
       <c r="A140" s="6" t="inlineStr">
         <is>
-          <t>Grupo AOC (Aníbal de Oliveira Cristina)</t>
+          <t>Grupo A. Silva &amp; Silva</t>
         </is>
       </c>
       <c r="B140" s="8" t="inlineStr">
@@ -6133,18 +6145,14 @@
         </is>
       </c>
       <c r="C140" s="8" t="inlineStr"/>
-      <c r="D140" s="6" t="inlineStr">
-        <is>
-          <t>Aníbal Cristina (fundador, 1990)</t>
-        </is>
-      </c>
+      <c r="D140" s="6" t="inlineStr"/>
       <c r="E140" s="6" t="inlineStr"/>
       <c r="F140" s="6" t="inlineStr"/>
       <c r="G140" s="6" t="inlineStr"/>
       <c r="H140" s="6" t="inlineStr"/>
       <c r="I140" s="8" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Seixal</t>
         </is>
       </c>
       <c r="J140" s="8" t="inlineStr">
@@ -6156,7 +6164,7 @@
     <row r="141" ht="26" customHeight="1">
       <c r="A141" s="6" t="inlineStr">
         <is>
-          <t>Grupo Mais Empresas / Construções Mais</t>
+          <t>Grupo André Guimarães (Portugal)</t>
         </is>
       </c>
       <c r="B141" s="8" t="inlineStr">
@@ -6165,30 +6173,26 @@
         </is>
       </c>
       <c r="C141" s="8" t="inlineStr"/>
-      <c r="D141" s="6" t="inlineStr"/>
+      <c r="D141" s="6" t="inlineStr">
+        <is>
+          <t>Fundador falecido· hoje liderado pelos filhos (Brasil), sem responsável PT confirmado</t>
+        </is>
+      </c>
       <c r="E141" s="6" t="inlineStr"/>
       <c r="F141" s="6" t="inlineStr"/>
       <c r="G141" s="6" t="inlineStr"/>
       <c r="H141" s="6" t="inlineStr">
         <is>
-          <t>grupomaisempresas.pt</t>
-        </is>
-      </c>
-      <c r="I141" s="8" t="inlineStr">
-        <is>
-          <t>Leiria</t>
-        </is>
-      </c>
-      <c r="J141" s="8" t="inlineStr">
-        <is>
-          <t>Leiria</t>
-        </is>
-      </c>
+          <t>andreguimaraes.com.br</t>
+        </is>
+      </c>
+      <c r="I141" s="8" t="inlineStr"/>
+      <c r="J141" s="8" t="inlineStr"/>
     </row>
     <row r="142" ht="26" customHeight="1">
       <c r="A142" s="6" t="inlineStr">
         <is>
-          <t>Grupo NB Portugal</t>
+          <t>Grupo André Jordan</t>
         </is>
       </c>
       <c r="B142" s="8" t="inlineStr">
@@ -6199,7 +6203,7 @@
       <c r="C142" s="8" t="inlineStr"/>
       <c r="D142" s="6" t="inlineStr">
         <is>
-          <t>Ioav Blanche (presidente)</t>
+          <t>Gilberto Jordan (CEO desde 2009 · sucede a André Jordan, falecido 2024)</t>
         </is>
       </c>
       <c r="E142" s="6" t="inlineStr"/>
@@ -6207,24 +6211,24 @@
       <c r="G142" s="6" t="inlineStr"/>
       <c r="H142" s="6" t="inlineStr">
         <is>
-          <t>gruponbportugal.pt</t>
+          <t>andrejordangroup.pt</t>
         </is>
       </c>
       <c r="I142" s="8" t="inlineStr">
         <is>
-          <t>Aveiro</t>
+          <t>Sintra</t>
         </is>
       </c>
       <c r="J142" s="8" t="inlineStr">
         <is>
-          <t>Aveiro</t>
+          <t>Lisboa</t>
         </is>
       </c>
     </row>
     <row r="143" ht="26" customHeight="1">
       <c r="A143" s="6" t="inlineStr">
         <is>
-          <t>Grupo Pestana (Pestana Residences)</t>
+          <t>Grupo AOC (Aníbal de Oliveira Cristina)</t>
         </is>
       </c>
       <c r="B143" s="8" t="inlineStr">
@@ -6235,20 +6239,16 @@
       <c r="C143" s="8" t="inlineStr"/>
       <c r="D143" s="6" t="inlineStr">
         <is>
-          <t>Dionísio Pestana (Chairman/dono)</t>
+          <t>Aníbal Cristina (fundador, 1990)</t>
         </is>
       </c>
       <c r="E143" s="6" t="inlineStr"/>
       <c r="F143" s="6" t="inlineStr"/>
       <c r="G143" s="6" t="inlineStr"/>
-      <c r="H143" s="6" t="inlineStr">
-        <is>
-          <t>pestana.com</t>
-        </is>
-      </c>
+      <c r="H143" s="6" t="inlineStr"/>
       <c r="I143" s="8" t="inlineStr">
         <is>
-          <t>Sines/Lagoa</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="J143" s="8" t="inlineStr">
@@ -6260,7 +6260,7 @@
     <row r="144" ht="26" customHeight="1">
       <c r="A144" s="6" t="inlineStr">
         <is>
-          <t>Hillside House Coimbra, Lda</t>
+          <t>Grupo Mais Empresas / Construções Mais</t>
         </is>
       </c>
       <c r="B144" s="8" t="inlineStr">
@@ -6275,24 +6275,24 @@
       <c r="G144" s="6" t="inlineStr"/>
       <c r="H144" s="6" t="inlineStr">
         <is>
-          <t>hillside.pt</t>
+          <t>grupomaisempresas.pt</t>
         </is>
       </c>
       <c r="I144" s="8" t="inlineStr">
         <is>
-          <t>Mealhada (projeto em Coimbra)</t>
+          <t>Leiria</t>
         </is>
       </c>
       <c r="J144" s="8" t="inlineStr">
         <is>
-          <t>Aveiro</t>
+          <t>Leiria</t>
         </is>
       </c>
     </row>
     <row r="145" ht="26" customHeight="1">
       <c r="A145" s="6" t="inlineStr">
         <is>
-          <t>Iconic Jeunesse, Unipessoal, Lda</t>
+          <t>Grupo NB Portugal</t>
         </is>
       </c>
       <c r="B145" s="8" t="inlineStr">
@@ -6301,30 +6301,34 @@
         </is>
       </c>
       <c r="C145" s="8" t="inlineStr"/>
-      <c r="D145" s="6" t="inlineStr"/>
+      <c r="D145" s="6" t="inlineStr">
+        <is>
+          <t>Ioav Blanche (presidente)</t>
+        </is>
+      </c>
       <c r="E145" s="6" t="inlineStr"/>
       <c r="F145" s="6" t="inlineStr"/>
       <c r="G145" s="6" t="inlineStr"/>
       <c r="H145" s="6" t="inlineStr">
         <is>
-          <t>zenithresidences.pt</t>
+          <t>gruponbportugal.pt</t>
         </is>
       </c>
       <c r="I145" s="8" t="inlineStr">
         <is>
-          <t>Portimão</t>
+          <t>Aveiro</t>
         </is>
       </c>
       <c r="J145" s="8" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Aveiro</t>
         </is>
       </c>
     </row>
     <row r="146" ht="26" customHeight="1">
       <c r="A146" s="6" t="inlineStr">
         <is>
-          <t>Invesquart – Real Estate Promotor</t>
+          <t>Grupo Pestana (Pestana Residences)</t>
         </is>
       </c>
       <c r="B146" s="8" t="inlineStr">
@@ -6333,26 +6337,34 @@
         </is>
       </c>
       <c r="C146" s="8" t="inlineStr"/>
-      <c r="D146" s="6" t="inlineStr"/>
+      <c r="D146" s="6" t="inlineStr">
+        <is>
+          <t>Dionísio Pestana (Chairman/dono)</t>
+        </is>
+      </c>
       <c r="E146" s="6" t="inlineStr"/>
       <c r="F146" s="6" t="inlineStr"/>
       <c r="G146" s="6" t="inlineStr"/>
-      <c r="H146" s="6" t="inlineStr"/>
+      <c r="H146" s="6" t="inlineStr">
+        <is>
+          <t>pestana.com</t>
+        </is>
+      </c>
       <c r="I146" s="8" t="inlineStr">
         <is>
-          <t>Loulé (Quarteira)</t>
+          <t>Sines/Lagoa</t>
         </is>
       </c>
       <c r="J146" s="8" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Setúbal</t>
         </is>
       </c>
     </row>
     <row r="147" ht="26" customHeight="1">
       <c r="A147" s="6" t="inlineStr">
         <is>
-          <t>Le Parc</t>
+          <t>Hillside House Coimbra, Lda</t>
         </is>
       </c>
       <c r="B147" s="8" t="inlineStr">
@@ -6367,24 +6379,24 @@
       <c r="G147" s="6" t="inlineStr"/>
       <c r="H147" s="6" t="inlineStr">
         <is>
-          <t>leparc.pt</t>
+          <t>hillside.pt</t>
         </is>
       </c>
       <c r="I147" s="8" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Mealhada (projeto em Coimbra)</t>
         </is>
       </c>
       <c r="J147" s="8" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Aveiro</t>
         </is>
       </c>
     </row>
     <row r="148" ht="26" customHeight="1">
       <c r="A148" s="6" t="inlineStr">
         <is>
-          <t>Lux Premium</t>
+          <t>Iconic Jeunesse, Unipessoal, Lda</t>
         </is>
       </c>
       <c r="B148" s="8" t="inlineStr">
@@ -6393,34 +6405,30 @@
         </is>
       </c>
       <c r="C148" s="8" t="inlineStr"/>
-      <c r="D148" s="6" t="inlineStr">
-        <is>
-          <t>Claude Berda (fundador)</t>
-        </is>
-      </c>
+      <c r="D148" s="6" t="inlineStr"/>
       <c r="E148" s="6" t="inlineStr"/>
       <c r="F148" s="6" t="inlineStr"/>
       <c r="G148" s="6" t="inlineStr"/>
       <c r="H148" s="6" t="inlineStr">
         <is>
-          <t>luxpremium.net</t>
+          <t>zenithresidences.pt</t>
         </is>
       </c>
       <c r="I148" s="8" t="inlineStr">
         <is>
-          <t>Coimbra</t>
+          <t>Portimão</t>
         </is>
       </c>
       <c r="J148" s="8" t="inlineStr">
         <is>
-          <t>Coimbra</t>
+          <t>Faro</t>
         </is>
       </c>
     </row>
     <row r="149" ht="26" customHeight="1">
       <c r="A149" s="6" t="inlineStr">
         <is>
-          <t>MAJA Construções, S.A.</t>
+          <t>Invesquart – Real Estate Promotor</t>
         </is>
       </c>
       <c r="B149" s="8" t="inlineStr">
@@ -6429,18 +6437,14 @@
         </is>
       </c>
       <c r="C149" s="8" t="inlineStr"/>
-      <c r="D149" s="6" t="inlineStr">
-        <is>
-          <t>Manuel António e Jorge Almeida (fundadores, 1972)</t>
-        </is>
-      </c>
+      <c r="D149" s="6" t="inlineStr"/>
       <c r="E149" s="6" t="inlineStr"/>
       <c r="F149" s="6" t="inlineStr"/>
       <c r="G149" s="6" t="inlineStr"/>
       <c r="H149" s="6" t="inlineStr"/>
       <c r="I149" s="8" t="inlineStr">
         <is>
-          <t>Albufeira</t>
+          <t>Loulé (Quarteira)</t>
         </is>
       </c>
       <c r="J149" s="8" t="inlineStr">
@@ -6452,7 +6456,7 @@
     <row r="150" ht="26" customHeight="1">
       <c r="A150" s="6" t="inlineStr">
         <is>
-          <t>Mariano Investe – Empreendimentos Imobiliários</t>
+          <t>Le Parc</t>
         </is>
       </c>
       <c r="B150" s="8" t="inlineStr">
@@ -6465,22 +6469,26 @@
       <c r="E150" s="6" t="inlineStr"/>
       <c r="F150" s="6" t="inlineStr"/>
       <c r="G150" s="6" t="inlineStr"/>
-      <c r="H150" s="6" t="inlineStr"/>
+      <c r="H150" s="6" t="inlineStr">
+        <is>
+          <t>leparc.pt</t>
+        </is>
+      </c>
       <c r="I150" s="8" t="inlineStr">
         <is>
-          <t>Santarém</t>
+          <t>Faro</t>
         </is>
       </c>
       <c r="J150" s="8" t="inlineStr">
         <is>
-          <t>Santarém</t>
+          <t>Faro</t>
         </is>
       </c>
     </row>
     <row r="151" ht="26" customHeight="1">
       <c r="A151" s="6" t="inlineStr">
         <is>
-          <t>Maven (Maven Invest)</t>
+          <t>Lux Premium</t>
         </is>
       </c>
       <c r="B151" s="8" t="inlineStr">
@@ -6491,7 +6499,7 @@
       <c r="C151" s="8" t="inlineStr"/>
       <c r="D151" s="6" t="inlineStr">
         <is>
-          <t>Yehonatan Gourvitch (CEO)</t>
+          <t>Claude Berda (fundador)</t>
         </is>
       </c>
       <c r="E151" s="6" t="inlineStr"/>
@@ -6499,24 +6507,24 @@
       <c r="G151" s="6" t="inlineStr"/>
       <c r="H151" s="6" t="inlineStr">
         <is>
-          <t>maveninvest.pt</t>
+          <t>luxpremium.net</t>
         </is>
       </c>
       <c r="I151" s="8" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Coimbra</t>
         </is>
       </c>
       <c r="J151" s="8" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Coimbra</t>
         </is>
       </c>
     </row>
     <row r="152" ht="26" customHeight="1">
       <c r="A152" s="6" t="inlineStr">
         <is>
-          <t>Máscarazul – Mediação Imobiliária, Lda</t>
+          <t>MAJA Construções, S.A.</t>
         </is>
       </c>
       <c r="B152" s="8" t="inlineStr">
@@ -6525,7 +6533,11 @@
         </is>
       </c>
       <c r="C152" s="8" t="inlineStr"/>
-      <c r="D152" s="6" t="inlineStr"/>
+      <c r="D152" s="6" t="inlineStr">
+        <is>
+          <t>Manuel António e Jorge Almeida (fundadores, 1972)</t>
+        </is>
+      </c>
       <c r="E152" s="6" t="inlineStr"/>
       <c r="F152" s="6" t="inlineStr"/>
       <c r="G152" s="6" t="inlineStr"/>
@@ -6544,7 +6556,7 @@
     <row r="153" ht="26" customHeight="1">
       <c r="A153" s="6" t="inlineStr">
         <is>
-          <t>Nova Atlantic</t>
+          <t>Mariano Investe – Empreendimentos Imobiliários</t>
         </is>
       </c>
       <c r="B153" s="8" t="inlineStr">
@@ -6553,30 +6565,26 @@
         </is>
       </c>
       <c r="C153" s="8" t="inlineStr"/>
-      <c r="D153" s="6" t="inlineStr">
-        <is>
-          <t>Matan Amitai (co-fundador)</t>
-        </is>
-      </c>
+      <c r="D153" s="6" t="inlineStr"/>
       <c r="E153" s="6" t="inlineStr"/>
       <c r="F153" s="6" t="inlineStr"/>
       <c r="G153" s="6" t="inlineStr"/>
       <c r="H153" s="6" t="inlineStr"/>
       <c r="I153" s="8" t="inlineStr">
         <is>
-          <t>Viana do Castelo</t>
+          <t>Santarém</t>
         </is>
       </c>
       <c r="J153" s="8" t="inlineStr">
         <is>
-          <t>Viana do Castelo</t>
+          <t>Santarém</t>
         </is>
       </c>
     </row>
     <row r="154" ht="26" customHeight="1">
       <c r="A154" s="6" t="inlineStr">
         <is>
-          <t>OCM Portugal (O'Connor Murphy)</t>
+          <t>Maven (Maven Invest)</t>
         </is>
       </c>
       <c r="B154" s="8" t="inlineStr">
@@ -6585,30 +6593,34 @@
         </is>
       </c>
       <c r="C154" s="8" t="inlineStr"/>
-      <c r="D154" s="6" t="inlineStr"/>
+      <c r="D154" s="6" t="inlineStr">
+        <is>
+          <t>Yehonatan Gourvitch (CEO)</t>
+        </is>
+      </c>
       <c r="E154" s="6" t="inlineStr"/>
       <c r="F154" s="6" t="inlineStr"/>
       <c r="G154" s="6" t="inlineStr"/>
       <c r="H154" s="6" t="inlineStr">
         <is>
-          <t>oconnormurphy.ie</t>
+          <t>maveninvest.pt</t>
         </is>
       </c>
       <c r="I154" s="8" t="inlineStr">
         <is>
-          <t>Olhão</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="J154" s="8" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Setúbal</t>
         </is>
       </c>
     </row>
     <row r="155" ht="26" customHeight="1">
       <c r="A155" s="6" t="inlineStr">
         <is>
-          <t>PATRIMOINIMMO PORTUGAL</t>
+          <t>Máscarazul – Mediação Imobiliária, Lda</t>
         </is>
       </c>
       <c r="B155" s="8" t="inlineStr">
@@ -6624,7 +6636,7 @@
       <c r="H155" s="6" t="inlineStr"/>
       <c r="I155" s="8" t="inlineStr">
         <is>
-          <t>Lagoa</t>
+          <t>Albufeira</t>
         </is>
       </c>
       <c r="J155" s="8" t="inlineStr">
@@ -6636,7 +6648,7 @@
     <row r="156" ht="26" customHeight="1">
       <c r="A156" s="6" t="inlineStr">
         <is>
-          <t>Pelicano – Investimento Imobiliário, S.A.</t>
+          <t>Nova Atlantic</t>
         </is>
       </c>
       <c r="B156" s="8" t="inlineStr">
@@ -6647,7 +6659,7 @@
       <c r="C156" s="8" t="inlineStr"/>
       <c r="D156" s="6" t="inlineStr">
         <is>
-          <t>Joaquim Da Cunha Mendes Duarte (Presidente) / Sergio Manuel Mendes Gomes (Administrador)</t>
+          <t>Matan Amitai (co-fundador)</t>
         </is>
       </c>
       <c r="E156" s="6" t="inlineStr"/>
@@ -6656,19 +6668,19 @@
       <c r="H156" s="6" t="inlineStr"/>
       <c r="I156" s="8" t="inlineStr">
         <is>
-          <t>Palmela</t>
+          <t>Viana do Castelo</t>
         </is>
       </c>
       <c r="J156" s="8" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Viana do Castelo</t>
         </is>
       </c>
     </row>
     <row r="157" ht="26" customHeight="1">
       <c r="A157" s="6" t="inlineStr">
         <is>
-          <t>Pensaplano</t>
+          <t>OCM Portugal (O'Connor Murphy)</t>
         </is>
       </c>
       <c r="B157" s="8" t="inlineStr">
@@ -6681,22 +6693,26 @@
       <c r="E157" s="6" t="inlineStr"/>
       <c r="F157" s="6" t="inlineStr"/>
       <c r="G157" s="6" t="inlineStr"/>
-      <c r="H157" s="6" t="inlineStr"/>
+      <c r="H157" s="6" t="inlineStr">
+        <is>
+          <t>oconnormurphy.ie</t>
+        </is>
+      </c>
       <c r="I157" s="8" t="inlineStr">
         <is>
-          <t>Coimbra</t>
+          <t>Olhão</t>
         </is>
       </c>
       <c r="J157" s="8" t="inlineStr">
         <is>
-          <t>Coimbra</t>
+          <t>Faro</t>
         </is>
       </c>
     </row>
     <row r="158" ht="26" customHeight="1">
       <c r="A158" s="6" t="inlineStr">
         <is>
-          <t>Portugal Slow Living</t>
+          <t>PATRIMOINIMMO PORTUGAL</t>
         </is>
       </c>
       <c r="B158" s="8" t="inlineStr">
@@ -6712,19 +6728,19 @@
       <c r="H158" s="6" t="inlineStr"/>
       <c r="I158" s="8" t="inlineStr">
         <is>
-          <t>Montijo</t>
+          <t>Lagoa</t>
         </is>
       </c>
       <c r="J158" s="8" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Faro</t>
         </is>
       </c>
     </row>
     <row r="159" ht="26" customHeight="1">
       <c r="A159" s="6" t="inlineStr">
         <is>
-          <t>Rivage Properties</t>
+          <t>Pelicano – Investimento Imobiliário, S.A.</t>
         </is>
       </c>
       <c r="B159" s="8" t="inlineStr">
@@ -6735,7 +6751,7 @@
       <c r="C159" s="8" t="inlineStr"/>
       <c r="D159" s="6" t="inlineStr">
         <is>
-          <t>João Ribeiro (CEO e fundador, com Jorge Duarte e Fernando Santos)</t>
+          <t>Joaquim Da Cunha Mendes Duarte (Presidente) / Sergio Manuel Mendes Gomes (Administrador)</t>
         </is>
       </c>
       <c r="E159" s="6" t="inlineStr"/>
@@ -6744,19 +6760,19 @@
       <c r="H159" s="6" t="inlineStr"/>
       <c r="I159" s="8" t="inlineStr">
         <is>
-          <t>Gondomar</t>
+          <t>Palmela</t>
         </is>
       </c>
       <c r="J159" s="8" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Setúbal</t>
         </is>
       </c>
     </row>
     <row r="160" ht="26" customHeight="1">
       <c r="A160" s="6" t="inlineStr">
         <is>
-          <t>Rodrigues &amp; Vermelho – Construções, S.A.</t>
+          <t>Pensaplano</t>
         </is>
       </c>
       <c r="B160" s="8" t="inlineStr">
@@ -6765,34 +6781,26 @@
         </is>
       </c>
       <c r="C160" s="8" t="inlineStr"/>
-      <c r="D160" s="6" t="inlineStr">
-        <is>
-          <t>Celestino Vermelho Rodrigues (contacto)</t>
-        </is>
-      </c>
+      <c r="D160" s="6" t="inlineStr"/>
       <c r="E160" s="6" t="inlineStr"/>
       <c r="F160" s="6" t="inlineStr"/>
       <c r="G160" s="6" t="inlineStr"/>
-      <c r="H160" s="6" t="inlineStr">
-        <is>
-          <t>rodriguesevermelho.com</t>
-        </is>
-      </c>
+      <c r="H160" s="6" t="inlineStr"/>
       <c r="I160" s="8" t="inlineStr">
         <is>
-          <t>Lagos</t>
+          <t>Coimbra</t>
         </is>
       </c>
       <c r="J160" s="8" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Coimbra</t>
         </is>
       </c>
     </row>
     <row r="161" ht="26" customHeight="1">
       <c r="A161" s="6" t="inlineStr">
         <is>
-          <t>SOLUM PROGRESS</t>
+          <t>Portugal Slow Living</t>
         </is>
       </c>
       <c r="B161" s="8" t="inlineStr">
@@ -6808,19 +6816,19 @@
       <c r="H161" s="6" t="inlineStr"/>
       <c r="I161" s="8" t="inlineStr">
         <is>
-          <t>Coimbra</t>
+          <t>Montijo</t>
         </is>
       </c>
       <c r="J161" s="8" t="inlineStr">
         <is>
-          <t>Coimbra</t>
+          <t>Setúbal</t>
         </is>
       </c>
     </row>
     <row r="162" ht="26" customHeight="1">
       <c r="A162" s="6" t="inlineStr">
         <is>
-          <t>Southshore Investments</t>
+          <t>Rivage Properties</t>
         </is>
       </c>
       <c r="B162" s="8" t="inlineStr">
@@ -6829,30 +6837,30 @@
         </is>
       </c>
       <c r="C162" s="8" t="inlineStr"/>
-      <c r="D162" s="6" t="inlineStr"/>
+      <c r="D162" s="6" t="inlineStr">
+        <is>
+          <t>João Ribeiro (CEO e fundador, com Jorge Duarte e Fernando Santos)</t>
+        </is>
+      </c>
       <c r="E162" s="6" t="inlineStr"/>
       <c r="F162" s="6" t="inlineStr"/>
       <c r="G162" s="6" t="inlineStr"/>
-      <c r="H162" s="6" t="inlineStr">
-        <is>
-          <t>southshoreinvest.com</t>
-        </is>
-      </c>
+      <c r="H162" s="6" t="inlineStr"/>
       <c r="I162" s="8" t="inlineStr">
         <is>
-          <t>Almada</t>
+          <t>Gondomar</t>
         </is>
       </c>
       <c r="J162" s="8" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Porto</t>
         </is>
       </c>
     </row>
     <row r="163" ht="26" customHeight="1">
       <c r="A163" s="6" t="inlineStr">
         <is>
-          <t>Terrace Benefit, Lda</t>
+          <t>Rodrigues &amp; Vermelho – Construções, S.A.</t>
         </is>
       </c>
       <c r="B163" s="8" t="inlineStr">
@@ -6861,14 +6869,22 @@
         </is>
       </c>
       <c r="C163" s="8" t="inlineStr"/>
-      <c r="D163" s="6" t="inlineStr"/>
+      <c r="D163" s="6" t="inlineStr">
+        <is>
+          <t>Celestino Vermelho Rodrigues (contacto)</t>
+        </is>
+      </c>
       <c r="E163" s="6" t="inlineStr"/>
       <c r="F163" s="6" t="inlineStr"/>
       <c r="G163" s="6" t="inlineStr"/>
-      <c r="H163" s="6" t="inlineStr"/>
+      <c r="H163" s="6" t="inlineStr">
+        <is>
+          <t>rodriguesevermelho.com</t>
+        </is>
+      </c>
       <c r="I163" s="8" t="inlineStr">
         <is>
-          <t>Loulé (Quarteira)</t>
+          <t>Lagos</t>
         </is>
       </c>
       <c r="J163" s="8" t="inlineStr">
@@ -6880,7 +6896,7 @@
     <row r="164" ht="26" customHeight="1">
       <c r="A164" s="6" t="inlineStr">
         <is>
-          <t>The Epic Group</t>
+          <t>SOLUM PROGRESS</t>
         </is>
       </c>
       <c r="B164" s="8" t="inlineStr">
@@ -6893,26 +6909,22 @@
       <c r="E164" s="6" t="inlineStr"/>
       <c r="F164" s="6" t="inlineStr"/>
       <c r="G164" s="6" t="inlineStr"/>
-      <c r="H164" s="6" t="inlineStr">
-        <is>
-          <t>valentavillas.com</t>
-        </is>
-      </c>
+      <c r="H164" s="6" t="inlineStr"/>
       <c r="I164" s="8" t="inlineStr">
         <is>
-          <t>Ílhavo</t>
+          <t>Coimbra</t>
         </is>
       </c>
       <c r="J164" s="8" t="inlineStr">
         <is>
-          <t>Aveiro</t>
+          <t>Coimbra</t>
         </is>
       </c>
     </row>
     <row r="165" ht="26" customHeight="1">
       <c r="A165" s="6" t="inlineStr">
         <is>
-          <t>Udra – Grupo San José</t>
+          <t>Southshore Investments</t>
         </is>
       </c>
       <c r="B165" s="8" t="inlineStr">
@@ -6925,10 +6937,14 @@
       <c r="E165" s="6" t="inlineStr"/>
       <c r="F165" s="6" t="inlineStr"/>
       <c r="G165" s="6" t="inlineStr"/>
-      <c r="H165" s="6" t="inlineStr"/>
+      <c r="H165" s="6" t="inlineStr">
+        <is>
+          <t>southshoreinvest.com</t>
+        </is>
+      </c>
       <c r="I165" s="8" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Almada</t>
         </is>
       </c>
       <c r="J165" s="8" t="inlineStr">
@@ -6940,7 +6956,7 @@
     <row r="166" ht="26" customHeight="1">
       <c r="A166" s="6" t="inlineStr">
         <is>
-          <t>Urban Green Private (UGP)</t>
+          <t>Terrace Benefit, Lda</t>
         </is>
       </c>
       <c r="B166" s="8" t="inlineStr">
@@ -6949,22 +6965,14 @@
         </is>
       </c>
       <c r="C166" s="8" t="inlineStr"/>
-      <c r="D166" s="6" t="inlineStr">
-        <is>
-          <t>Thomas Coughlan (fundador)</t>
-        </is>
-      </c>
+      <c r="D166" s="6" t="inlineStr"/>
       <c r="E166" s="6" t="inlineStr"/>
       <c r="F166" s="6" t="inlineStr"/>
       <c r="G166" s="6" t="inlineStr"/>
-      <c r="H166" s="6" t="inlineStr">
-        <is>
-          <t>ugp.ie</t>
-        </is>
-      </c>
+      <c r="H166" s="6" t="inlineStr"/>
       <c r="I166" s="8" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Loulé (Quarteira)</t>
         </is>
       </c>
       <c r="J166" s="8" t="inlineStr">
@@ -6976,7 +6984,7 @@
     <row r="167" ht="26" customHeight="1">
       <c r="A167" s="6" t="inlineStr">
         <is>
-          <t>Urban Office</t>
+          <t>The Epic Group</t>
         </is>
       </c>
       <c r="B167" s="8" t="inlineStr">
@@ -6991,24 +6999,24 @@
       <c r="G167" s="6" t="inlineStr"/>
       <c r="H167" s="6" t="inlineStr">
         <is>
-          <t>urbanoffice.pt</t>
+          <t>valentavillas.com</t>
         </is>
       </c>
       <c r="I167" s="8" t="inlineStr">
         <is>
-          <t>Torres Vedras</t>
+          <t>Ílhavo</t>
         </is>
       </c>
       <c r="J167" s="8" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Aveiro</t>
         </is>
       </c>
     </row>
     <row r="168" ht="26" customHeight="1">
       <c r="A168" s="6" t="inlineStr">
         <is>
-          <t>Vale do Lobo Resort</t>
+          <t>Udra – Grupo San José</t>
         </is>
       </c>
       <c r="B168" s="8" t="inlineStr">
@@ -7021,26 +7029,22 @@
       <c r="E168" s="6" t="inlineStr"/>
       <c r="F168" s="6" t="inlineStr"/>
       <c r="G168" s="6" t="inlineStr"/>
-      <c r="H168" s="6" t="inlineStr">
-        <is>
-          <t>valedolobo.com</t>
-        </is>
-      </c>
+      <c r="H168" s="6" t="inlineStr"/>
       <c r="I168" s="8" t="inlineStr">
         <is>
-          <t>Loulé</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="J168" s="8" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Setúbal</t>
         </is>
       </c>
     </row>
     <row r="169" ht="26" customHeight="1">
       <c r="A169" s="6" t="inlineStr">
         <is>
-          <t>Vila Galé</t>
+          <t>Urban Green Private (UGP)</t>
         </is>
       </c>
       <c r="B169" s="8" t="inlineStr">
@@ -7049,21 +7053,121 @@
         </is>
       </c>
       <c r="C169" s="8" t="inlineStr"/>
-      <c r="D169" s="6" t="inlineStr"/>
+      <c r="D169" s="6" t="inlineStr">
+        <is>
+          <t>Thomas Coughlan (fundador)</t>
+        </is>
+      </c>
       <c r="E169" s="6" t="inlineStr"/>
       <c r="F169" s="6" t="inlineStr"/>
       <c r="G169" s="6" t="inlineStr"/>
       <c r="H169" s="6" t="inlineStr">
         <is>
+          <t>ugp.ie</t>
+        </is>
+      </c>
+      <c r="I169" s="8" t="inlineStr">
+        <is>
+          <t>Faro</t>
+        </is>
+      </c>
+      <c r="J169" s="8" t="inlineStr">
+        <is>
+          <t>Faro</t>
+        </is>
+      </c>
+    </row>
+    <row r="170" ht="26" customHeight="1">
+      <c r="A170" s="6" t="inlineStr">
+        <is>
+          <t>Urban Office</t>
+        </is>
+      </c>
+      <c r="B170" s="8" t="inlineStr">
+        <is>
+          <t>Nao</t>
+        </is>
+      </c>
+      <c r="C170" s="8" t="inlineStr"/>
+      <c r="D170" s="6" t="inlineStr"/>
+      <c r="E170" s="6" t="inlineStr"/>
+      <c r="F170" s="6" t="inlineStr"/>
+      <c r="G170" s="6" t="inlineStr"/>
+      <c r="H170" s="6" t="inlineStr">
+        <is>
+          <t>urbanoffice.pt</t>
+        </is>
+      </c>
+      <c r="I170" s="8" t="inlineStr">
+        <is>
+          <t>Torres Vedras</t>
+        </is>
+      </c>
+      <c r="J170" s="8" t="inlineStr">
+        <is>
+          <t>Lisboa</t>
+        </is>
+      </c>
+    </row>
+    <row r="171" ht="26" customHeight="1">
+      <c r="A171" s="6" t="inlineStr">
+        <is>
+          <t>Vale do Lobo Resort</t>
+        </is>
+      </c>
+      <c r="B171" s="8" t="inlineStr">
+        <is>
+          <t>Nao</t>
+        </is>
+      </c>
+      <c r="C171" s="8" t="inlineStr"/>
+      <c r="D171" s="6" t="inlineStr"/>
+      <c r="E171" s="6" t="inlineStr"/>
+      <c r="F171" s="6" t="inlineStr"/>
+      <c r="G171" s="6" t="inlineStr"/>
+      <c r="H171" s="6" t="inlineStr">
+        <is>
+          <t>valedolobo.com</t>
+        </is>
+      </c>
+      <c r="I171" s="8" t="inlineStr">
+        <is>
+          <t>Loulé</t>
+        </is>
+      </c>
+      <c r="J171" s="8" t="inlineStr">
+        <is>
+          <t>Faro</t>
+        </is>
+      </c>
+    </row>
+    <row r="172" ht="26" customHeight="1">
+      <c r="A172" s="6" t="inlineStr">
+        <is>
+          <t>Vila Galé</t>
+        </is>
+      </c>
+      <c r="B172" s="8" t="inlineStr">
+        <is>
+          <t>Nao</t>
+        </is>
+      </c>
+      <c r="C172" s="8" t="inlineStr"/>
+      <c r="D172" s="6" t="inlineStr"/>
+      <c r="E172" s="6" t="inlineStr"/>
+      <c r="F172" s="6" t="inlineStr"/>
+      <c r="G172" s="6" t="inlineStr"/>
+      <c r="H172" s="6" t="inlineStr">
+        <is>
           <t>vilagale.com</t>
         </is>
       </c>
-      <c r="I169" s="8" t="inlineStr">
+      <c r="I172" s="8" t="inlineStr">
         <is>
           <t>Golegã</t>
         </is>
       </c>
-      <c r="J169" s="8" t="inlineStr">
+      <c r="J172" s="8" t="inlineStr">
         <is>
           <t>Santarém</t>
         </is>
@@ -7117,19 +7221,19 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E71" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E72" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E73" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E87" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E88" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E89" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E106" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E107" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E108" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E109" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E110" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E111" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E112" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E113" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E114" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E115" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E88" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E89" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E90" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E109" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E110" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E111" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E112" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E113" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E114" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E115" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E116" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E117" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E118" r:id="rId59"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
@@ -7170,7 +7274,7 @@
         </is>
       </c>
       <c r="B2" s="11" t="n">
-        <v>168</v>
+        <v>171</v>
       </c>
     </row>
     <row r="3">
@@ -7180,7 +7284,7 @@
         </is>
       </c>
       <c r="B3" s="11" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="4">
@@ -7190,7 +7294,7 @@
         </is>
       </c>
       <c r="B4" s="11" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="5">
@@ -7200,7 +7304,7 @@
         </is>
       </c>
       <c r="B5" s="11" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="6">
@@ -7230,7 +7334,7 @@
         </is>
       </c>
       <c r="B8" s="11" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
Add Groundfloor and JCKL Portugal (173 total)
Found via the 2025 edition of the Prémio Nacional do Imobiliário
finalists list. Also folds newly found projects into three existing
entries: Krest Investments (Horizon Ocean Gardens), Teixeira Duarte
Real Estate (Fábrica 1921).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SRBJwGmSsYkTHKJbGCM5ca
</commit_message>
<xml_diff>
--- a/Lista_Contactos.xlsx
+++ b/Lista_Contactos.xlsx
@@ -203,8 +203,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Contactos" displayName="Contactos" ref="A1:J172" headerRowCount="1">
-  <autoFilter ref="A1:J172"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Contactos" displayName="Contactos" ref="A1:J174" headerRowCount="1">
+  <autoFilter ref="A1:J174"/>
   <tableColumns count="10">
     <tableColumn id="1" name="Nome da Empresa"/>
     <tableColumn id="2" name="Prioritario"/>
@@ -510,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J172"/>
+  <dimension ref="A1:J174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4624,7 +4624,7 @@
     <row r="94" ht="26" customHeight="1">
       <c r="A94" s="6" t="inlineStr">
         <is>
-          <t>Hines Portugal</t>
+          <t>Groundfloor – Premium Investments</t>
         </is>
       </c>
       <c r="B94" s="7" t="inlineStr">
@@ -4633,17 +4633,13 @@
         </is>
       </c>
       <c r="C94" s="8" t="inlineStr"/>
-      <c r="D94" s="6" t="inlineStr">
-        <is>
-          <t>Vanessa Gelado (Senior Managing Director, Head of Southern Europe)</t>
-        </is>
-      </c>
+      <c r="D94" s="6" t="inlineStr"/>
       <c r="E94" s="6" t="inlineStr"/>
       <c r="F94" s="6" t="inlineStr"/>
       <c r="G94" s="6" t="inlineStr"/>
       <c r="H94" s="6" t="inlineStr">
         <is>
-          <t>hines.com</t>
+          <t>theartt.pt</t>
         </is>
       </c>
       <c r="I94" s="8" t="inlineStr">
@@ -4660,7 +4656,7 @@
     <row r="95" ht="26" customHeight="1">
       <c r="A95" s="6" t="inlineStr">
         <is>
-          <t>Imolote</t>
+          <t>Hines Portugal</t>
         </is>
       </c>
       <c r="B95" s="7" t="inlineStr">
@@ -4671,7 +4667,7 @@
       <c r="C95" s="8" t="inlineStr"/>
       <c r="D95" s="6" t="inlineStr">
         <is>
-          <t>Paulo Vaz Ferreira (sócio e CEO desde 2019, confiança moderada)</t>
+          <t>Vanessa Gelado (Senior Managing Director, Head of Southern Europe)</t>
         </is>
       </c>
       <c r="E95" s="6" t="inlineStr"/>
@@ -4679,24 +4675,24 @@
       <c r="G95" s="6" t="inlineStr"/>
       <c r="H95" s="6" t="inlineStr">
         <is>
-          <t>imolote.pt</t>
+          <t>hines.com</t>
         </is>
       </c>
       <c r="I95" s="8" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="J95" s="8" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Lisboa</t>
         </is>
       </c>
     </row>
     <row r="96" ht="26" customHeight="1">
       <c r="A96" s="6" t="inlineStr">
         <is>
-          <t>João Magalhães &amp; Alexandre Magalhães (promotores individuais)</t>
+          <t>Imolote</t>
         </is>
       </c>
       <c r="B96" s="7" t="inlineStr">
@@ -4707,13 +4703,17 @@
       <c r="C96" s="8" t="inlineStr"/>
       <c r="D96" s="6" t="inlineStr">
         <is>
-          <t>João Magalhães e Alexandre Magalhães (promotores individuais)</t>
+          <t>Paulo Vaz Ferreira (sócio e CEO desde 2019, confiança moderada)</t>
         </is>
       </c>
       <c r="E96" s="6" t="inlineStr"/>
       <c r="F96" s="6" t="inlineStr"/>
       <c r="G96" s="6" t="inlineStr"/>
-      <c r="H96" s="6" t="inlineStr"/>
+      <c r="H96" s="6" t="inlineStr">
+        <is>
+          <t>imolote.pt</t>
+        </is>
+      </c>
       <c r="I96" s="8" t="inlineStr">
         <is>
           <t>Porto</t>
@@ -4728,7 +4728,7 @@
     <row r="97" ht="26" customHeight="1">
       <c r="A97" s="6" t="inlineStr">
         <is>
-          <t>KKR Imo, S.A.</t>
+          <t>JCKL Portugal – Investimentos Imobiliários</t>
         </is>
       </c>
       <c r="B97" s="7" t="inlineStr">
@@ -4737,11 +4737,7 @@
         </is>
       </c>
       <c r="C97" s="8" t="inlineStr"/>
-      <c r="D97" s="6" t="inlineStr">
-        <is>
-          <t>Vera Kendall (administradora, dados de 2018 · confiança baixa)</t>
-        </is>
-      </c>
+      <c r="D97" s="6" t="inlineStr"/>
       <c r="E97" s="6" t="inlineStr"/>
       <c r="F97" s="6" t="inlineStr"/>
       <c r="G97" s="6" t="inlineStr"/>
@@ -4760,7 +4756,7 @@
     <row r="98" ht="26" customHeight="1">
       <c r="A98" s="6" t="inlineStr">
         <is>
-          <t>Neptune Developments</t>
+          <t>João Magalhães &amp; Alexandre Magalhães (promotores individuais)</t>
         </is>
       </c>
       <c r="B98" s="7" t="inlineStr">
@@ -4769,30 +4765,30 @@
         </is>
       </c>
       <c r="C98" s="8" t="inlineStr"/>
-      <c r="D98" s="6" t="inlineStr"/>
+      <c r="D98" s="6" t="inlineStr">
+        <is>
+          <t>João Magalhães e Alexandre Magalhães (promotores individuais)</t>
+        </is>
+      </c>
       <c r="E98" s="6" t="inlineStr"/>
       <c r="F98" s="6" t="inlineStr"/>
       <c r="G98" s="6" t="inlineStr"/>
-      <c r="H98" s="6" t="inlineStr">
-        <is>
-          <t>neptune-developments.com</t>
-        </is>
-      </c>
+      <c r="H98" s="6" t="inlineStr"/>
       <c r="I98" s="8" t="inlineStr">
         <is>
-          <t>Cascais</t>
+          <t>Porto</t>
         </is>
       </c>
       <c r="J98" s="8" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Porto</t>
         </is>
       </c>
     </row>
     <row r="99" ht="26" customHeight="1">
       <c r="A99" s="6" t="inlineStr">
         <is>
-          <t>Onyria Group</t>
+          <t>KKR Imo, S.A.</t>
         </is>
       </c>
       <c r="B99" s="7" t="inlineStr">
@@ -4803,20 +4799,16 @@
       <c r="C99" s="8" t="inlineStr"/>
       <c r="D99" s="6" t="inlineStr">
         <is>
-          <t>José Carlos Pinto Coelho (fundador, 1986)</t>
+          <t>Vera Kendall (administradora, dados de 2018 · confiança baixa)</t>
         </is>
       </c>
       <c r="E99" s="6" t="inlineStr"/>
       <c r="F99" s="6" t="inlineStr"/>
       <c r="G99" s="6" t="inlineStr"/>
-      <c r="H99" s="6" t="inlineStr">
-        <is>
-          <t>onyriagroup.com</t>
-        </is>
-      </c>
+      <c r="H99" s="6" t="inlineStr"/>
       <c r="I99" s="8" t="inlineStr">
         <is>
-          <t>Cascais</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="J99" s="8" t="inlineStr">
@@ -4828,7 +4820,7 @@
     <row r="100" ht="26" customHeight="1">
       <c r="A100" s="6" t="inlineStr">
         <is>
-          <t>Portaviv</t>
+          <t>Neptune Developments</t>
         </is>
       </c>
       <c r="B100" s="7" t="inlineStr">
@@ -4837,30 +4829,30 @@
         </is>
       </c>
       <c r="C100" s="8" t="inlineStr"/>
-      <c r="D100" s="6" t="inlineStr">
-        <is>
-          <t>Nuno Cunha (Managing Director)</t>
-        </is>
-      </c>
+      <c r="D100" s="6" t="inlineStr"/>
       <c r="E100" s="6" t="inlineStr"/>
       <c r="F100" s="6" t="inlineStr"/>
       <c r="G100" s="6" t="inlineStr"/>
-      <c r="H100" s="6" t="inlineStr"/>
+      <c r="H100" s="6" t="inlineStr">
+        <is>
+          <t>neptune-developments.com</t>
+        </is>
+      </c>
       <c r="I100" s="8" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Cascais</t>
         </is>
       </c>
       <c r="J100" s="8" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Lisboa</t>
         </is>
       </c>
     </row>
     <row r="101" ht="26" customHeight="1">
       <c r="A101" s="6" t="inlineStr">
         <is>
-          <t>REABILITA</t>
+          <t>Onyria Group</t>
         </is>
       </c>
       <c r="B101" s="7" t="inlineStr">
@@ -4869,18 +4861,22 @@
         </is>
       </c>
       <c r="C101" s="8" t="inlineStr"/>
-      <c r="D101" s="6" t="inlineStr"/>
+      <c r="D101" s="6" t="inlineStr">
+        <is>
+          <t>José Carlos Pinto Coelho (fundador, 1986)</t>
+        </is>
+      </c>
       <c r="E101" s="6" t="inlineStr"/>
       <c r="F101" s="6" t="inlineStr"/>
       <c r="G101" s="6" t="inlineStr"/>
       <c r="H101" s="6" t="inlineStr">
         <is>
-          <t>reabilita.pt</t>
+          <t>onyriagroup.com</t>
         </is>
       </c>
       <c r="I101" s="8" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Cascais</t>
         </is>
       </c>
       <c r="J101" s="8" t="inlineStr">
@@ -4892,7 +4888,7 @@
     <row r="102" ht="26" customHeight="1">
       <c r="A102" s="6" t="inlineStr">
         <is>
-          <t>REDASSET</t>
+          <t>Portaviv</t>
         </is>
       </c>
       <c r="B102" s="7" t="inlineStr">
@@ -4901,26 +4897,30 @@
         </is>
       </c>
       <c r="C102" s="8" t="inlineStr"/>
-      <c r="D102" s="6" t="inlineStr"/>
+      <c r="D102" s="6" t="inlineStr">
+        <is>
+          <t>Nuno Cunha (Managing Director)</t>
+        </is>
+      </c>
       <c r="E102" s="6" t="inlineStr"/>
       <c r="F102" s="6" t="inlineStr"/>
       <c r="G102" s="6" t="inlineStr"/>
       <c r="H102" s="6" t="inlineStr"/>
       <c r="I102" s="8" t="inlineStr">
         <is>
-          <t>Amadora</t>
+          <t>Porto</t>
         </is>
       </c>
       <c r="J102" s="8" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Porto</t>
         </is>
       </c>
     </row>
     <row r="103" ht="26" customHeight="1">
       <c r="A103" s="6" t="inlineStr">
         <is>
-          <t>RM Promo (JV M2O Group / RJB Home)</t>
+          <t>REABILITA</t>
         </is>
       </c>
       <c r="B103" s="7" t="inlineStr">
@@ -4933,22 +4933,26 @@
       <c r="E103" s="6" t="inlineStr"/>
       <c r="F103" s="6" t="inlineStr"/>
       <c r="G103" s="6" t="inlineStr"/>
-      <c r="H103" s="6" t="inlineStr"/>
+      <c r="H103" s="6" t="inlineStr">
+        <is>
+          <t>reabilita.pt</t>
+        </is>
+      </c>
       <c r="I103" s="8" t="inlineStr">
         <is>
-          <t>Matosinhos</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="J103" s="8" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Lisboa</t>
         </is>
       </c>
     </row>
     <row r="104" ht="26" customHeight="1">
       <c r="A104" s="6" t="inlineStr">
         <is>
-          <t>Selicomi Portugal (Victoria Group)</t>
+          <t>REDASSET</t>
         </is>
       </c>
       <c r="B104" s="7" t="inlineStr">
@@ -4964,7 +4968,7 @@
       <c r="H104" s="6" t="inlineStr"/>
       <c r="I104" s="8" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Amadora</t>
         </is>
       </c>
       <c r="J104" s="8" t="inlineStr">
@@ -4976,7 +4980,7 @@
     <row r="105" ht="26" customHeight="1">
       <c r="A105" s="6" t="inlineStr">
         <is>
-          <t>SGAL – Sociedade Gestora da Alta de Lisboa</t>
+          <t>RM Promo (JV M2O Group / RJB Home)</t>
         </is>
       </c>
       <c r="B105" s="7" t="inlineStr">
@@ -4989,26 +4993,22 @@
       <c r="E105" s="6" t="inlineStr"/>
       <c r="F105" s="6" t="inlineStr"/>
       <c r="G105" s="6" t="inlineStr"/>
-      <c r="H105" s="6" t="inlineStr">
-        <is>
-          <t>altadelisboa.com</t>
-        </is>
-      </c>
+      <c r="H105" s="6" t="inlineStr"/>
       <c r="I105" s="8" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Matosinhos</t>
         </is>
       </c>
       <c r="J105" s="8" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Porto</t>
         </is>
       </c>
     </row>
     <row r="106" ht="26" customHeight="1">
       <c r="A106" s="6" t="inlineStr">
         <is>
-          <t>Shalu Investments</t>
+          <t>Selicomi Portugal (Victoria Group)</t>
         </is>
       </c>
       <c r="B106" s="7" t="inlineStr">
@@ -5017,34 +5017,26 @@
         </is>
       </c>
       <c r="C106" s="8" t="inlineStr"/>
-      <c r="D106" s="6" t="inlineStr">
-        <is>
-          <t>Itai Fridman (Founder &amp; Managing Director)</t>
-        </is>
-      </c>
+      <c r="D106" s="6" t="inlineStr"/>
       <c r="E106" s="6" t="inlineStr"/>
       <c r="F106" s="6" t="inlineStr"/>
       <c r="G106" s="6" t="inlineStr"/>
-      <c r="H106" s="6" t="inlineStr">
-        <is>
-          <t>shaluinvest.pt</t>
-        </is>
-      </c>
+      <c r="H106" s="6" t="inlineStr"/>
       <c r="I106" s="8" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="J106" s="8" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Lisboa</t>
         </is>
       </c>
     </row>
     <row r="107" ht="26" customHeight="1">
       <c r="A107" s="6" t="inlineStr">
         <is>
-          <t>Square Asset Management</t>
+          <t>SGAL – Sociedade Gestora da Alta de Lisboa</t>
         </is>
       </c>
       <c r="B107" s="7" t="inlineStr">
@@ -5059,7 +5051,7 @@
       <c r="G107" s="6" t="inlineStr"/>
       <c r="H107" s="6" t="inlineStr">
         <is>
-          <t>squaream.pt</t>
+          <t>altadelisboa.com</t>
         </is>
       </c>
       <c r="I107" s="8" t="inlineStr">
@@ -5076,7 +5068,7 @@
     <row r="108" ht="26" customHeight="1">
       <c r="A108" s="6" t="inlineStr">
         <is>
-          <t>Taga Urbanic</t>
+          <t>Shalu Investments</t>
         </is>
       </c>
       <c r="B108" s="7" t="inlineStr">
@@ -5085,14 +5077,22 @@
         </is>
       </c>
       <c r="C108" s="8" t="inlineStr"/>
-      <c r="D108" s="6" t="inlineStr"/>
+      <c r="D108" s="6" t="inlineStr">
+        <is>
+          <t>Itai Fridman (Founder &amp; Managing Director)</t>
+        </is>
+      </c>
       <c r="E108" s="6" t="inlineStr"/>
       <c r="F108" s="6" t="inlineStr"/>
       <c r="G108" s="6" t="inlineStr"/>
-      <c r="H108" s="6" t="inlineStr"/>
+      <c r="H108" s="6" t="inlineStr">
+        <is>
+          <t>shaluinvest.pt</t>
+        </is>
+      </c>
       <c r="I108" s="8" t="inlineStr">
         <is>
-          <t>Maia</t>
+          <t>Porto</t>
         </is>
       </c>
       <c r="J108" s="8" t="inlineStr">
@@ -5104,31 +5104,27 @@
     <row r="109" ht="26" customHeight="1">
       <c r="A109" s="6" t="inlineStr">
         <is>
-          <t>Amorim Luxury</t>
-        </is>
-      </c>
-      <c r="B109" s="8" t="inlineStr">
-        <is>
-          <t>Nao</t>
+          <t>Square Asset Management</t>
+        </is>
+      </c>
+      <c r="B109" s="7" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
       <c r="C109" s="8" t="inlineStr"/>
-      <c r="D109" s="6" t="inlineStr">
-        <is>
-          <t>Miguel Guedes de Sousa (Founder &amp; CEO)</t>
-        </is>
-      </c>
-      <c r="E109" s="9" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/miguelguedesdesousa/</t>
-        </is>
-      </c>
+      <c r="D109" s="6" t="inlineStr"/>
+      <c r="E109" s="6" t="inlineStr"/>
       <c r="F109" s="6" t="inlineStr"/>
       <c r="G109" s="6" t="inlineStr"/>
-      <c r="H109" s="6" t="inlineStr"/>
+      <c r="H109" s="6" t="inlineStr">
+        <is>
+          <t>squaream.pt</t>
+        </is>
+      </c>
       <c r="I109" s="8" t="inlineStr">
         <is>
-          <t>Lisboa/Grândola/Lagoa</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="J109" s="8" t="inlineStr">
@@ -5140,43 +5136,35 @@
     <row r="110" ht="26" customHeight="1">
       <c r="A110" s="6" t="inlineStr">
         <is>
-          <t>Emblezart</t>
-        </is>
-      </c>
-      <c r="B110" s="8" t="inlineStr">
-        <is>
-          <t>Nao</t>
+          <t>Taga Urbanic</t>
+        </is>
+      </c>
+      <c r="B110" s="7" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
       <c r="C110" s="8" t="inlineStr"/>
-      <c r="D110" s="6" t="inlineStr">
-        <is>
-          <t>David Faria (CEO e sócio único)</t>
-        </is>
-      </c>
-      <c r="E110" s="9" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/david-faria-a301a466/</t>
-        </is>
-      </c>
+      <c r="D110" s="6" t="inlineStr"/>
+      <c r="E110" s="6" t="inlineStr"/>
       <c r="F110" s="6" t="inlineStr"/>
       <c r="G110" s="6" t="inlineStr"/>
       <c r="H110" s="6" t="inlineStr"/>
       <c r="I110" s="8" t="inlineStr">
         <is>
-          <t>Guimarães</t>
+          <t>Maia</t>
         </is>
       </c>
       <c r="J110" s="8" t="inlineStr">
         <is>
-          <t>Braga</t>
+          <t>Porto</t>
         </is>
       </c>
     </row>
     <row r="111" ht="26" customHeight="1">
       <c r="A111" s="6" t="inlineStr">
         <is>
-          <t>Grupo Azinor</t>
+          <t>Amorim Luxury</t>
         </is>
       </c>
       <c r="B111" s="8" t="inlineStr">
@@ -5187,12 +5175,12 @@
       <c r="C111" s="8" t="inlineStr"/>
       <c r="D111" s="6" t="inlineStr">
         <is>
-          <t>Carlos Silva Neves (administrador)</t>
+          <t>Miguel Guedes de Sousa (Founder &amp; CEO)</t>
         </is>
       </c>
       <c r="E111" s="9" t="inlineStr">
         <is>
-          <t>https://pt.linkedin.com/in/carlos-silva-neves-3b0711142</t>
+          <t>https://www.linkedin.com/in/miguelguedesdesousa/</t>
         </is>
       </c>
       <c r="F111" s="6" t="inlineStr"/>
@@ -5200,7 +5188,7 @@
       <c r="H111" s="6" t="inlineStr"/>
       <c r="I111" s="8" t="inlineStr">
         <is>
-          <t>Oeiras</t>
+          <t>Lisboa/Grândola/Lagoa</t>
         </is>
       </c>
       <c r="J111" s="8" t="inlineStr">
@@ -5212,7 +5200,7 @@
     <row r="112" ht="26" customHeight="1">
       <c r="A112" s="6" t="inlineStr">
         <is>
-          <t>JPAIVA Investimentos / JPAIVA Engenharia e Construção</t>
+          <t>Emblezart</t>
         </is>
       </c>
       <c r="B112" s="8" t="inlineStr">
@@ -5223,36 +5211,32 @@
       <c r="C112" s="8" t="inlineStr"/>
       <c r="D112" s="6" t="inlineStr">
         <is>
-          <t>Igor Castro (CEO)</t>
+          <t>David Faria (CEO e sócio único)</t>
         </is>
       </c>
       <c r="E112" s="9" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/igor-castro-a0026b22b/</t>
+          <t>https://www.linkedin.com/in/david-faria-a301a466/</t>
         </is>
       </c>
       <c r="F112" s="6" t="inlineStr"/>
       <c r="G112" s="6" t="inlineStr"/>
-      <c r="H112" s="6" t="inlineStr">
-        <is>
-          <t>jpaiva.pt</t>
-        </is>
-      </c>
+      <c r="H112" s="6" t="inlineStr"/>
       <c r="I112" s="8" t="inlineStr">
         <is>
-          <t>Coimbra</t>
+          <t>Guimarães</t>
         </is>
       </c>
       <c r="J112" s="8" t="inlineStr">
         <is>
-          <t>Coimbra</t>
+          <t>Braga</t>
         </is>
       </c>
     </row>
     <row r="113" ht="26" customHeight="1">
       <c r="A113" s="6" t="inlineStr">
         <is>
-          <t>Mello RDC</t>
+          <t>Grupo Azinor</t>
         </is>
       </c>
       <c r="B113" s="8" t="inlineStr">
@@ -5263,36 +5247,32 @@
       <c r="C113" s="8" t="inlineStr"/>
       <c r="D113" s="6" t="inlineStr">
         <is>
-          <t>António Ribeiro da Cunha (CEO)</t>
+          <t>Carlos Silva Neves (administrador)</t>
         </is>
       </c>
       <c r="E113" s="9" t="inlineStr">
         <is>
-          <t>https://pt.linkedin.com/in/ant%C3%B3nio-ribeiro-da-cunha-77b974112</t>
+          <t>https://pt.linkedin.com/in/carlos-silva-neves-3b0711142</t>
         </is>
       </c>
       <c r="F113" s="6" t="inlineStr"/>
       <c r="G113" s="6" t="inlineStr"/>
-      <c r="H113" s="6" t="inlineStr">
-        <is>
-          <t>mellordc.pt</t>
-        </is>
-      </c>
+      <c r="H113" s="6" t="inlineStr"/>
       <c r="I113" s="8" t="inlineStr">
         <is>
-          <t>Grândola (Melides)</t>
+          <t>Oeiras</t>
         </is>
       </c>
       <c r="J113" s="8" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Lisboa</t>
         </is>
       </c>
     </row>
     <row r="114" ht="26" customHeight="1">
       <c r="A114" s="6" t="inlineStr">
         <is>
-          <t>Ombria Resort (Grupo Pontos)</t>
+          <t>JPAIVA Investimentos / JPAIVA Engenharia e Construção</t>
         </is>
       </c>
       <c r="B114" s="8" t="inlineStr">
@@ -5303,36 +5283,36 @@
       <c r="C114" s="8" t="inlineStr"/>
       <c r="D114" s="6" t="inlineStr">
         <is>
-          <t>Patrick Freeman (CEO Ombria desde 2023)· CEO do Grupo Pontos é Timo Kokkila</t>
+          <t>Igor Castro (CEO)</t>
         </is>
       </c>
       <c r="E114" s="9" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/patricksfreeman/</t>
+          <t>https://www.linkedin.com/in/igor-castro-a0026b22b/</t>
         </is>
       </c>
       <c r="F114" s="6" t="inlineStr"/>
       <c r="G114" s="6" t="inlineStr"/>
       <c r="H114" s="6" t="inlineStr">
         <is>
-          <t>ombria.com</t>
+          <t>jpaiva.pt</t>
         </is>
       </c>
       <c r="I114" s="8" t="inlineStr">
         <is>
-          <t>Loulé</t>
+          <t>Coimbra</t>
         </is>
       </c>
       <c r="J114" s="8" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Coimbra</t>
         </is>
       </c>
     </row>
     <row r="115" ht="26" customHeight="1">
       <c r="A115" s="6" t="inlineStr">
         <is>
-          <t>Soccal &amp; Vaz Invest</t>
+          <t>Mello RDC</t>
         </is>
       </c>
       <c r="B115" s="8" t="inlineStr">
@@ -5343,24 +5323,24 @@
       <c r="C115" s="8" t="inlineStr"/>
       <c r="D115" s="6" t="inlineStr">
         <is>
-          <t>António Vaz (fundador e CEO)</t>
+          <t>António Ribeiro da Cunha (CEO)</t>
         </is>
       </c>
       <c r="E115" s="9" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/antonio-vaz-9444998a/</t>
+          <t>https://pt.linkedin.com/in/ant%C3%B3nio-ribeiro-da-cunha-77b974112</t>
         </is>
       </c>
       <c r="F115" s="6" t="inlineStr"/>
       <c r="G115" s="6" t="inlineStr"/>
       <c r="H115" s="6" t="inlineStr">
         <is>
-          <t>soccal-vaz.com</t>
+          <t>mellordc.pt</t>
         </is>
       </c>
       <c r="I115" s="8" t="inlineStr">
         <is>
-          <t>Sines</t>
+          <t>Grândola (Melides)</t>
         </is>
       </c>
       <c r="J115" s="8" t="inlineStr">
@@ -5372,7 +5352,7 @@
     <row r="116" ht="26" customHeight="1">
       <c r="A116" s="6" t="inlineStr">
         <is>
-          <t>Solid Sentinel</t>
+          <t>Ombria Resort (Grupo Pontos)</t>
         </is>
       </c>
       <c r="B116" s="8" t="inlineStr">
@@ -5383,36 +5363,36 @@
       <c r="C116" s="8" t="inlineStr"/>
       <c r="D116" s="6" t="inlineStr">
         <is>
-          <t>Alain Gross (Co-Founder e CEO)</t>
+          <t>Patrick Freeman (CEO Ombria desde 2023)· CEO do Grupo Pontos é Timo Kokkila</t>
         </is>
       </c>
       <c r="E116" s="9" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/alain-gross-3351411/</t>
+          <t>https://www.linkedin.com/in/patricksfreeman/</t>
         </is>
       </c>
       <c r="F116" s="6" t="inlineStr"/>
       <c r="G116" s="6" t="inlineStr"/>
       <c r="H116" s="6" t="inlineStr">
         <is>
-          <t>solidsentinel.pt</t>
+          <t>ombria.com</t>
         </is>
       </c>
       <c r="I116" s="8" t="inlineStr">
         <is>
-          <t>Barreiro</t>
+          <t>Loulé</t>
         </is>
       </c>
       <c r="J116" s="8" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Faro</t>
         </is>
       </c>
     </row>
     <row r="117" ht="26" customHeight="1">
       <c r="A117" s="6" t="inlineStr">
         <is>
-          <t>Sonae Sierra</t>
+          <t>Soccal &amp; Vaz Invest</t>
         </is>
       </c>
       <c r="B117" s="8" t="inlineStr">
@@ -5423,36 +5403,36 @@
       <c r="C117" s="8" t="inlineStr"/>
       <c r="D117" s="6" t="inlineStr">
         <is>
-          <t>Fernando Guedes de Oliveira (CEO)</t>
+          <t>António Vaz (fundador e CEO)</t>
         </is>
       </c>
       <c r="E117" s="9" t="inlineStr">
         <is>
-          <t>https://pt.linkedin.com/in/fernando-oliveira-9622b817</t>
+          <t>https://www.linkedin.com/in/antonio-vaz-9444998a/</t>
         </is>
       </c>
       <c r="F117" s="6" t="inlineStr"/>
       <c r="G117" s="6" t="inlineStr"/>
       <c r="H117" s="6" t="inlineStr">
         <is>
-          <t>sonaesierra.com</t>
+          <t>soccal-vaz.com</t>
         </is>
       </c>
       <c r="I117" s="8" t="inlineStr">
         <is>
-          <t>Lisboa/Porto</t>
+          <t>Sines</t>
         </is>
       </c>
       <c r="J117" s="8" t="inlineStr">
         <is>
-          <t>nacional</t>
+          <t>Setúbal</t>
         </is>
       </c>
     </row>
     <row r="118" ht="26" customHeight="1">
       <c r="A118" s="6" t="inlineStr">
         <is>
-          <t>Square View</t>
+          <t>Solid Sentinel</t>
         </is>
       </c>
       <c r="B118" s="8" t="inlineStr">
@@ -5463,36 +5443,36 @@
       <c r="C118" s="8" t="inlineStr"/>
       <c r="D118" s="6" t="inlineStr">
         <is>
-          <t>Luis Horta e Costa (CEO/Fundador)</t>
+          <t>Alain Gross (Co-Founder e CEO)</t>
         </is>
       </c>
       <c r="E118" s="9" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/luis-horta-e-costa-377552241/</t>
+          <t>https://www.linkedin.com/in/alain-gross-3351411/</t>
         </is>
       </c>
       <c r="F118" s="6" t="inlineStr"/>
       <c r="G118" s="6" t="inlineStr"/>
       <c r="H118" s="6" t="inlineStr">
         <is>
-          <t>squareview.pt</t>
+          <t>solidsentinel.pt</t>
         </is>
       </c>
       <c r="I118" s="8" t="inlineStr">
         <is>
-          <t>Lisboa/Ericeira/Melides</t>
+          <t>Barreiro</t>
         </is>
       </c>
       <c r="J118" s="8" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Setúbal</t>
         </is>
       </c>
     </row>
     <row r="119" ht="26" customHeight="1">
       <c r="A119" s="6" t="inlineStr">
         <is>
-          <t>Algarve Property Shops</t>
+          <t>Sonae Sierra</t>
         </is>
       </c>
       <c r="B119" s="8" t="inlineStr">
@@ -5501,26 +5481,38 @@
         </is>
       </c>
       <c r="C119" s="8" t="inlineStr"/>
-      <c r="D119" s="6" t="inlineStr"/>
-      <c r="E119" s="6" t="inlineStr"/>
+      <c r="D119" s="6" t="inlineStr">
+        <is>
+          <t>Fernando Guedes de Oliveira (CEO)</t>
+        </is>
+      </c>
+      <c r="E119" s="9" t="inlineStr">
+        <is>
+          <t>https://pt.linkedin.com/in/fernando-oliveira-9622b817</t>
+        </is>
+      </c>
       <c r="F119" s="6" t="inlineStr"/>
       <c r="G119" s="6" t="inlineStr"/>
-      <c r="H119" s="6" t="inlineStr"/>
+      <c r="H119" s="6" t="inlineStr">
+        <is>
+          <t>sonaesierra.com</t>
+        </is>
+      </c>
       <c r="I119" s="8" t="inlineStr">
         <is>
-          <t>Tavira</t>
+          <t>Lisboa/Porto</t>
         </is>
       </c>
       <c r="J119" s="8" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>nacional</t>
         </is>
       </c>
     </row>
     <row r="120" ht="26" customHeight="1">
       <c r="A120" s="6" t="inlineStr">
         <is>
-          <t>Aresta Vitalicia</t>
+          <t>Square View</t>
         </is>
       </c>
       <c r="B120" s="8" t="inlineStr">
@@ -5529,26 +5521,38 @@
         </is>
       </c>
       <c r="C120" s="8" t="inlineStr"/>
-      <c r="D120" s="6" t="inlineStr"/>
-      <c r="E120" s="6" t="inlineStr"/>
+      <c r="D120" s="6" t="inlineStr">
+        <is>
+          <t>Luis Horta e Costa (CEO/Fundador)</t>
+        </is>
+      </c>
+      <c r="E120" s="9" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/luis-horta-e-costa-377552241/</t>
+        </is>
+      </c>
       <c r="F120" s="6" t="inlineStr"/>
       <c r="G120" s="6" t="inlineStr"/>
-      <c r="H120" s="6" t="inlineStr"/>
+      <c r="H120" s="6" t="inlineStr">
+        <is>
+          <t>squareview.pt</t>
+        </is>
+      </c>
       <c r="I120" s="8" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Lisboa/Ericeira/Melides</t>
         </is>
       </c>
       <c r="J120" s="8" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Lisboa</t>
         </is>
       </c>
     </row>
     <row r="121" ht="26" customHeight="1">
       <c r="A121" s="6" t="inlineStr">
         <is>
-          <t>Arrow Global Portugal</t>
+          <t>Algarve Property Shops</t>
         </is>
       </c>
       <c r="B121" s="8" t="inlineStr">
@@ -5557,18 +5561,14 @@
         </is>
       </c>
       <c r="C121" s="8" t="inlineStr"/>
-      <c r="D121" s="6" t="inlineStr">
-        <is>
-          <t>João Bugalho (CEO)</t>
-        </is>
-      </c>
+      <c r="D121" s="6" t="inlineStr"/>
       <c r="E121" s="6" t="inlineStr"/>
       <c r="F121" s="6" t="inlineStr"/>
       <c r="G121" s="6" t="inlineStr"/>
       <c r="H121" s="6" t="inlineStr"/>
       <c r="I121" s="8" t="inlineStr">
         <is>
-          <t>Loulé (Almancil/Quinta do Lago)</t>
+          <t>Tavira</t>
         </is>
       </c>
       <c r="J121" s="8" t="inlineStr">
@@ -5580,7 +5580,7 @@
     <row r="122" ht="26" customHeight="1">
       <c r="A122" s="6" t="inlineStr">
         <is>
-          <t>Baltor – Engenharia e Construção</t>
+          <t>Aresta Vitalicia</t>
         </is>
       </c>
       <c r="B122" s="8" t="inlineStr">
@@ -5589,22 +5589,14 @@
         </is>
       </c>
       <c r="C122" s="8" t="inlineStr"/>
-      <c r="D122" s="6" t="inlineStr">
-        <is>
-          <t>Paulo Balinha e Bruno Torres (fundadores, 2008)</t>
-        </is>
-      </c>
+      <c r="D122" s="6" t="inlineStr"/>
       <c r="E122" s="6" t="inlineStr"/>
       <c r="F122" s="6" t="inlineStr"/>
       <c r="G122" s="6" t="inlineStr"/>
-      <c r="H122" s="6" t="inlineStr">
-        <is>
-          <t>baltor.pt</t>
-        </is>
-      </c>
+      <c r="H122" s="6" t="inlineStr"/>
       <c r="I122" s="8" t="inlineStr">
         <is>
-          <t>Setúbal (sede Viana do Castelo)</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="J122" s="8" t="inlineStr">
@@ -5616,7 +5608,7 @@
     <row r="123" ht="26" customHeight="1">
       <c r="A123" s="6" t="inlineStr">
         <is>
-          <t>Bond Group</t>
+          <t>Arrow Global Portugal</t>
         </is>
       </c>
       <c r="B123" s="8" t="inlineStr">
@@ -5625,26 +5617,30 @@
         </is>
       </c>
       <c r="C123" s="8" t="inlineStr"/>
-      <c r="D123" s="6" t="inlineStr"/>
+      <c r="D123" s="6" t="inlineStr">
+        <is>
+          <t>João Bugalho (CEO)</t>
+        </is>
+      </c>
       <c r="E123" s="6" t="inlineStr"/>
       <c r="F123" s="6" t="inlineStr"/>
       <c r="G123" s="6" t="inlineStr"/>
       <c r="H123" s="6" t="inlineStr"/>
       <c r="I123" s="8" t="inlineStr">
         <is>
-          <t>Amares</t>
+          <t>Loulé (Almancil/Quinta do Lago)</t>
         </is>
       </c>
       <c r="J123" s="8" t="inlineStr">
         <is>
-          <t>Braga</t>
+          <t>Faro</t>
         </is>
       </c>
     </row>
     <row r="124" ht="26" customHeight="1">
       <c r="A124" s="6" t="inlineStr">
         <is>
-          <t>Branco Real Estate</t>
+          <t>Baltor – Engenharia e Construção</t>
         </is>
       </c>
       <c r="B124" s="8" t="inlineStr">
@@ -5653,26 +5649,34 @@
         </is>
       </c>
       <c r="C124" s="8" t="inlineStr"/>
-      <c r="D124" s="6" t="inlineStr"/>
+      <c r="D124" s="6" t="inlineStr">
+        <is>
+          <t>Paulo Balinha e Bruno Torres (fundadores, 2008)</t>
+        </is>
+      </c>
       <c r="E124" s="6" t="inlineStr"/>
       <c r="F124" s="6" t="inlineStr"/>
       <c r="G124" s="6" t="inlineStr"/>
-      <c r="H124" s="6" t="inlineStr"/>
+      <c r="H124" s="6" t="inlineStr">
+        <is>
+          <t>baltor.pt</t>
+        </is>
+      </c>
       <c r="I124" s="8" t="inlineStr">
         <is>
-          <t>Lagos</t>
+          <t>Setúbal (sede Viana do Castelo)</t>
         </is>
       </c>
       <c r="J124" s="8" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Setúbal</t>
         </is>
       </c>
     </row>
     <row r="125" ht="26" customHeight="1">
       <c r="A125" s="6" t="inlineStr">
         <is>
-          <t>Casas do Sotavento</t>
+          <t>Bond Group</t>
         </is>
       </c>
       <c r="B125" s="8" t="inlineStr">
@@ -5685,26 +5689,22 @@
       <c r="E125" s="6" t="inlineStr"/>
       <c r="F125" s="6" t="inlineStr"/>
       <c r="G125" s="6" t="inlineStr"/>
-      <c r="H125" s="6" t="inlineStr">
-        <is>
-          <t>casasdosotavento.pt</t>
-        </is>
-      </c>
+      <c r="H125" s="6" t="inlineStr"/>
       <c r="I125" s="8" t="inlineStr">
         <is>
-          <t>Tavira</t>
+          <t>Amares</t>
         </is>
       </c>
       <c r="J125" s="8" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Braga</t>
         </is>
       </c>
     </row>
     <row r="126" ht="26" customHeight="1">
       <c r="A126" s="6" t="inlineStr">
         <is>
-          <t>Confidential Sphere – Investimento Imobiliário</t>
+          <t>Branco Real Estate</t>
         </is>
       </c>
       <c r="B126" s="8" t="inlineStr">
@@ -5720,7 +5720,7 @@
       <c r="H126" s="6" t="inlineStr"/>
       <c r="I126" s="8" t="inlineStr">
         <is>
-          <t>Silves</t>
+          <t>Lagos</t>
         </is>
       </c>
       <c r="J126" s="8" t="inlineStr">
@@ -5732,7 +5732,7 @@
     <row r="127" ht="26" customHeight="1">
       <c r="A127" s="6" t="inlineStr">
         <is>
-          <t>CS Ribeiro</t>
+          <t>Casas do Sotavento</t>
         </is>
       </c>
       <c r="B127" s="8" t="inlineStr">
@@ -5745,22 +5745,26 @@
       <c r="E127" s="6" t="inlineStr"/>
       <c r="F127" s="6" t="inlineStr"/>
       <c r="G127" s="6" t="inlineStr"/>
-      <c r="H127" s="6" t="inlineStr"/>
+      <c r="H127" s="6" t="inlineStr">
+        <is>
+          <t>casasdosotavento.pt</t>
+        </is>
+      </c>
       <c r="I127" s="8" t="inlineStr">
         <is>
-          <t>Guarda (atua Viseu/Coimbra)</t>
+          <t>Tavira</t>
         </is>
       </c>
       <c r="J127" s="8" t="inlineStr">
         <is>
-          <t>Guarda</t>
+          <t>Faro</t>
         </is>
       </c>
     </row>
     <row r="128" ht="26" customHeight="1">
       <c r="A128" s="6" t="inlineStr">
         <is>
-          <t>Discovery Land Company</t>
+          <t>Confidential Sphere – Investimento Imobiliário</t>
         </is>
       </c>
       <c r="B128" s="8" t="inlineStr">
@@ -5773,26 +5777,22 @@
       <c r="E128" s="6" t="inlineStr"/>
       <c r="F128" s="6" t="inlineStr"/>
       <c r="G128" s="6" t="inlineStr"/>
-      <c r="H128" s="6" t="inlineStr">
-        <is>
-          <t>discoverylandco.com</t>
-        </is>
-      </c>
+      <c r="H128" s="6" t="inlineStr"/>
       <c r="I128" s="8" t="inlineStr">
         <is>
-          <t>Grândola (Melides)</t>
+          <t>Silves</t>
         </is>
       </c>
       <c r="J128" s="8" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Faro</t>
         </is>
       </c>
     </row>
     <row r="129" ht="26" customHeight="1">
       <c r="A129" s="6" t="inlineStr">
         <is>
-          <t>DUJA – Sociedade de Construções, Lda</t>
+          <t>CS Ribeiro</t>
         </is>
       </c>
       <c r="B129" s="8" t="inlineStr">
@@ -5808,19 +5808,19 @@
       <c r="H129" s="6" t="inlineStr"/>
       <c r="I129" s="8" t="inlineStr">
         <is>
-          <t>Tavira</t>
+          <t>Guarda (atua Viseu/Coimbra)</t>
         </is>
       </c>
       <c r="J129" s="8" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Guarda</t>
         </is>
       </c>
     </row>
     <row r="130" ht="26" customHeight="1">
       <c r="A130" s="6" t="inlineStr">
         <is>
-          <t>Encobarra</t>
+          <t>Discovery Land Company</t>
         </is>
       </c>
       <c r="B130" s="8" t="inlineStr">
@@ -5829,30 +5829,30 @@
         </is>
       </c>
       <c r="C130" s="8" t="inlineStr"/>
-      <c r="D130" s="6" t="inlineStr">
-        <is>
-          <t>Aristides Alferes (administrador)</t>
-        </is>
-      </c>
+      <c r="D130" s="6" t="inlineStr"/>
       <c r="E130" s="6" t="inlineStr"/>
       <c r="F130" s="6" t="inlineStr"/>
       <c r="G130" s="6" t="inlineStr"/>
-      <c r="H130" s="6" t="inlineStr"/>
+      <c r="H130" s="6" t="inlineStr">
+        <is>
+          <t>discoverylandco.com</t>
+        </is>
+      </c>
       <c r="I130" s="8" t="inlineStr">
         <is>
-          <t>Aveiro (Aradas)</t>
+          <t>Grândola (Melides)</t>
         </is>
       </c>
       <c r="J130" s="8" t="inlineStr">
         <is>
-          <t>Aveiro</t>
+          <t>Setúbal</t>
         </is>
       </c>
     </row>
     <row r="131" ht="26" customHeight="1">
       <c r="A131" s="6" t="inlineStr">
         <is>
-          <t>Estrutural Group</t>
+          <t>DUJA – Sociedade de Construções, Lda</t>
         </is>
       </c>
       <c r="B131" s="8" t="inlineStr">
@@ -5861,30 +5861,26 @@
         </is>
       </c>
       <c r="C131" s="8" t="inlineStr"/>
-      <c r="D131" s="6" t="inlineStr">
-        <is>
-          <t>Hugo Mendes Pinto (Managing Partner)</t>
-        </is>
-      </c>
+      <c r="D131" s="6" t="inlineStr"/>
       <c r="E131" s="6" t="inlineStr"/>
       <c r="F131" s="6" t="inlineStr"/>
       <c r="G131" s="6" t="inlineStr"/>
       <c r="H131" s="6" t="inlineStr"/>
       <c r="I131" s="8" t="inlineStr">
         <is>
-          <t>Vila Franca de Xira</t>
+          <t>Tavira</t>
         </is>
       </c>
       <c r="J131" s="8" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Faro</t>
         </is>
       </c>
     </row>
     <row r="132" ht="26" customHeight="1">
       <c r="A132" s="6" t="inlineStr">
         <is>
-          <t>Explorer Investments (Explorer Real Estate)</t>
+          <t>Encobarra</t>
         </is>
       </c>
       <c r="B132" s="8" t="inlineStr">
@@ -5895,32 +5891,28 @@
       <c r="C132" s="8" t="inlineStr"/>
       <c r="D132" s="6" t="inlineStr">
         <is>
-          <t>Elizabeth Rothfield (CEO, Founding Partner)</t>
+          <t>Aristides Alferes (administrador)</t>
         </is>
       </c>
       <c r="E132" s="6" t="inlineStr"/>
       <c r="F132" s="6" t="inlineStr"/>
       <c r="G132" s="6" t="inlineStr"/>
-      <c r="H132" s="6" t="inlineStr">
-        <is>
-          <t>explorerinvestments.com</t>
-        </is>
-      </c>
+      <c r="H132" s="6" t="inlineStr"/>
       <c r="I132" s="8" t="inlineStr">
         <is>
-          <t>Sintra</t>
+          <t>Aveiro (Aradas)</t>
         </is>
       </c>
       <c r="J132" s="8" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Aveiro</t>
         </is>
       </c>
     </row>
     <row r="133" ht="26" customHeight="1">
       <c r="A133" s="6" t="inlineStr">
         <is>
-          <t>Finangeste, S.A.</t>
+          <t>Estrutural Group</t>
         </is>
       </c>
       <c r="B133" s="8" t="inlineStr">
@@ -5931,7 +5923,7 @@
       <c r="C133" s="8" t="inlineStr"/>
       <c r="D133" s="6" t="inlineStr">
         <is>
-          <t>Paul Henri Schelfhout (Presidente do CA) / Armando Lacerda Queiroz (administrador)</t>
+          <t>Hugo Mendes Pinto (Managing Partner)</t>
         </is>
       </c>
       <c r="E133" s="6" t="inlineStr"/>
@@ -5940,19 +5932,19 @@
       <c r="H133" s="6" t="inlineStr"/>
       <c r="I133" s="8" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Vila Franca de Xira</t>
         </is>
       </c>
       <c r="J133" s="8" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Lisboa</t>
         </is>
       </c>
     </row>
     <row r="134" ht="26" customHeight="1">
       <c r="A134" s="6" t="inlineStr">
         <is>
-          <t>FourPromo, Lda (Grupo M2O)</t>
+          <t>Explorer Investments (Explorer Real Estate)</t>
         </is>
       </c>
       <c r="B134" s="8" t="inlineStr">
@@ -5961,26 +5953,34 @@
         </is>
       </c>
       <c r="C134" s="8" t="inlineStr"/>
-      <c r="D134" s="6" t="inlineStr"/>
+      <c r="D134" s="6" t="inlineStr">
+        <is>
+          <t>Elizabeth Rothfield (CEO, Founding Partner)</t>
+        </is>
+      </c>
       <c r="E134" s="6" t="inlineStr"/>
       <c r="F134" s="6" t="inlineStr"/>
       <c r="G134" s="6" t="inlineStr"/>
-      <c r="H134" s="6" t="inlineStr"/>
+      <c r="H134" s="6" t="inlineStr">
+        <is>
+          <t>explorerinvestments.com</t>
+        </is>
+      </c>
       <c r="I134" s="8" t="inlineStr">
         <is>
-          <t>Loulé (Vilamoura)</t>
+          <t>Sintra</t>
         </is>
       </c>
       <c r="J134" s="8" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Lisboa</t>
         </is>
       </c>
     </row>
     <row r="135" ht="26" customHeight="1">
       <c r="A135" s="6" t="inlineStr">
         <is>
-          <t>Foz Gala Investments</t>
+          <t>Finangeste, S.A.</t>
         </is>
       </c>
       <c r="B135" s="8" t="inlineStr">
@@ -5989,26 +5989,30 @@
         </is>
       </c>
       <c r="C135" s="8" t="inlineStr"/>
-      <c r="D135" s="6" t="inlineStr"/>
+      <c r="D135" s="6" t="inlineStr">
+        <is>
+          <t>Paul Henri Schelfhout (Presidente do CA) / Armando Lacerda Queiroz (administrador)</t>
+        </is>
+      </c>
       <c r="E135" s="6" t="inlineStr"/>
       <c r="F135" s="6" t="inlineStr"/>
       <c r="G135" s="6" t="inlineStr"/>
       <c r="H135" s="6" t="inlineStr"/>
       <c r="I135" s="8" t="inlineStr">
         <is>
-          <t>Figueira da Foz</t>
+          <t>Faro</t>
         </is>
       </c>
       <c r="J135" s="8" t="inlineStr">
         <is>
-          <t>Coimbra</t>
+          <t>Faro</t>
         </is>
       </c>
     </row>
     <row r="136" ht="26" customHeight="1">
       <c r="A136" s="6" t="inlineStr">
         <is>
-          <t>Galvana Investimentos Imobiliários e Turísticos, Lda</t>
+          <t>FourPromo, Lda (Grupo M2O)</t>
         </is>
       </c>
       <c r="B136" s="8" t="inlineStr">
@@ -6024,7 +6028,7 @@
       <c r="H136" s="6" t="inlineStr"/>
       <c r="I136" s="8" t="inlineStr">
         <is>
-          <t>Albufeira</t>
+          <t>Loulé (Vilamoura)</t>
         </is>
       </c>
       <c r="J136" s="8" t="inlineStr">
@@ -6036,7 +6040,7 @@
     <row r="137" ht="26" customHeight="1">
       <c r="A137" s="6" t="inlineStr">
         <is>
-          <t>Genuino Investments</t>
+          <t>Foz Gala Investments</t>
         </is>
       </c>
       <c r="B137" s="8" t="inlineStr">
@@ -6049,26 +6053,22 @@
       <c r="E137" s="6" t="inlineStr"/>
       <c r="F137" s="6" t="inlineStr"/>
       <c r="G137" s="6" t="inlineStr"/>
-      <c r="H137" s="6" t="inlineStr">
-        <is>
-          <t>genuinoinvestments.com</t>
-        </is>
-      </c>
+      <c r="H137" s="6" t="inlineStr"/>
       <c r="I137" s="8" t="inlineStr">
         <is>
-          <t>Portimão</t>
+          <t>Figueira da Foz</t>
         </is>
       </c>
       <c r="J137" s="8" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Coimbra</t>
         </is>
       </c>
     </row>
     <row r="138" ht="26" customHeight="1">
       <c r="A138" s="6" t="inlineStr">
         <is>
-          <t>GFH (Grupo Ferreira Holding) / Ferreira Build Power (marca BeLiving)</t>
+          <t>Galvana Investimentos Imobiliários e Turísticos, Lda</t>
         </is>
       </c>
       <c r="B138" s="8" t="inlineStr">
@@ -6077,22 +6077,14 @@
         </is>
       </c>
       <c r="C138" s="8" t="inlineStr"/>
-      <c r="D138" s="6" t="inlineStr">
-        <is>
-          <t>Joaquim Silva (CEO Ferreira Build Power)</t>
-        </is>
-      </c>
+      <c r="D138" s="6" t="inlineStr"/>
       <c r="E138" s="6" t="inlineStr"/>
       <c r="F138" s="6" t="inlineStr"/>
       <c r="G138" s="6" t="inlineStr"/>
-      <c r="H138" s="6" t="inlineStr">
-        <is>
-          <t>ferreirabuildpower.com</t>
-        </is>
-      </c>
+      <c r="H138" s="6" t="inlineStr"/>
       <c r="I138" s="8" t="inlineStr">
         <is>
-          <t>Faro/Loulé</t>
+          <t>Albufeira</t>
         </is>
       </c>
       <c r="J138" s="8" t="inlineStr">
@@ -6104,7 +6096,7 @@
     <row r="139" ht="26" customHeight="1">
       <c r="A139" s="6" t="inlineStr">
         <is>
-          <t>Glowing</t>
+          <t>Genuino Investments</t>
         </is>
       </c>
       <c r="B139" s="8" t="inlineStr">
@@ -6119,24 +6111,24 @@
       <c r="G139" s="6" t="inlineStr"/>
       <c r="H139" s="6" t="inlineStr">
         <is>
-          <t>glowing.pt</t>
+          <t>genuinoinvestments.com</t>
         </is>
       </c>
       <c r="I139" s="8" t="inlineStr">
         <is>
-          <t>Alcácer do Sal</t>
+          <t>Portimão</t>
         </is>
       </c>
       <c r="J139" s="8" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Faro</t>
         </is>
       </c>
     </row>
     <row r="140" ht="26" customHeight="1">
       <c r="A140" s="6" t="inlineStr">
         <is>
-          <t>Grupo A. Silva &amp; Silva</t>
+          <t>GFH (Grupo Ferreira Holding) / Ferreira Build Power (marca BeLiving)</t>
         </is>
       </c>
       <c r="B140" s="8" t="inlineStr">
@@ -6145,26 +6137,34 @@
         </is>
       </c>
       <c r="C140" s="8" t="inlineStr"/>
-      <c r="D140" s="6" t="inlineStr"/>
+      <c r="D140" s="6" t="inlineStr">
+        <is>
+          <t>Joaquim Silva (CEO Ferreira Build Power)</t>
+        </is>
+      </c>
       <c r="E140" s="6" t="inlineStr"/>
       <c r="F140" s="6" t="inlineStr"/>
       <c r="G140" s="6" t="inlineStr"/>
-      <c r="H140" s="6" t="inlineStr"/>
+      <c r="H140" s="6" t="inlineStr">
+        <is>
+          <t>ferreirabuildpower.com</t>
+        </is>
+      </c>
       <c r="I140" s="8" t="inlineStr">
         <is>
-          <t>Seixal</t>
+          <t>Faro/Loulé</t>
         </is>
       </c>
       <c r="J140" s="8" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Faro</t>
         </is>
       </c>
     </row>
     <row r="141" ht="26" customHeight="1">
       <c r="A141" s="6" t="inlineStr">
         <is>
-          <t>Grupo André Guimarães (Portugal)</t>
+          <t>Glowing</t>
         </is>
       </c>
       <c r="B141" s="8" t="inlineStr">
@@ -6173,26 +6173,30 @@
         </is>
       </c>
       <c r="C141" s="8" t="inlineStr"/>
-      <c r="D141" s="6" t="inlineStr">
-        <is>
-          <t>Fundador falecido· hoje liderado pelos filhos (Brasil), sem responsável PT confirmado</t>
-        </is>
-      </c>
+      <c r="D141" s="6" t="inlineStr"/>
       <c r="E141" s="6" t="inlineStr"/>
       <c r="F141" s="6" t="inlineStr"/>
       <c r="G141" s="6" t="inlineStr"/>
       <c r="H141" s="6" t="inlineStr">
         <is>
-          <t>andreguimaraes.com.br</t>
-        </is>
-      </c>
-      <c r="I141" s="8" t="inlineStr"/>
-      <c r="J141" s="8" t="inlineStr"/>
+          <t>glowing.pt</t>
+        </is>
+      </c>
+      <c r="I141" s="8" t="inlineStr">
+        <is>
+          <t>Alcácer do Sal</t>
+        </is>
+      </c>
+      <c r="J141" s="8" t="inlineStr">
+        <is>
+          <t>Setúbal</t>
+        </is>
+      </c>
     </row>
     <row r="142" ht="26" customHeight="1">
       <c r="A142" s="6" t="inlineStr">
         <is>
-          <t>Grupo André Jordan</t>
+          <t>Grupo A. Silva &amp; Silva</t>
         </is>
       </c>
       <c r="B142" s="8" t="inlineStr">
@@ -6201,34 +6205,26 @@
         </is>
       </c>
       <c r="C142" s="8" t="inlineStr"/>
-      <c r="D142" s="6" t="inlineStr">
-        <is>
-          <t>Gilberto Jordan (CEO desde 2009 · sucede a André Jordan, falecido 2024)</t>
-        </is>
-      </c>
+      <c r="D142" s="6" t="inlineStr"/>
       <c r="E142" s="6" t="inlineStr"/>
       <c r="F142" s="6" t="inlineStr"/>
       <c r="G142" s="6" t="inlineStr"/>
-      <c r="H142" s="6" t="inlineStr">
-        <is>
-          <t>andrejordangroup.pt</t>
-        </is>
-      </c>
+      <c r="H142" s="6" t="inlineStr"/>
       <c r="I142" s="8" t="inlineStr">
         <is>
-          <t>Sintra</t>
+          <t>Seixal</t>
         </is>
       </c>
       <c r="J142" s="8" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Setúbal</t>
         </is>
       </c>
     </row>
     <row r="143" ht="26" customHeight="1">
       <c r="A143" s="6" t="inlineStr">
         <is>
-          <t>Grupo AOC (Aníbal de Oliveira Cristina)</t>
+          <t>Grupo André Guimarães (Portugal)</t>
         </is>
       </c>
       <c r="B143" s="8" t="inlineStr">
@@ -6239,28 +6235,24 @@
       <c r="C143" s="8" t="inlineStr"/>
       <c r="D143" s="6" t="inlineStr">
         <is>
-          <t>Aníbal Cristina (fundador, 1990)</t>
+          <t>Fundador falecido· hoje liderado pelos filhos (Brasil), sem responsável PT confirmado</t>
         </is>
       </c>
       <c r="E143" s="6" t="inlineStr"/>
       <c r="F143" s="6" t="inlineStr"/>
       <c r="G143" s="6" t="inlineStr"/>
-      <c r="H143" s="6" t="inlineStr"/>
-      <c r="I143" s="8" t="inlineStr">
-        <is>
-          <t>Setúbal</t>
-        </is>
-      </c>
-      <c r="J143" s="8" t="inlineStr">
-        <is>
-          <t>Setúbal</t>
-        </is>
-      </c>
+      <c r="H143" s="6" t="inlineStr">
+        <is>
+          <t>andreguimaraes.com.br</t>
+        </is>
+      </c>
+      <c r="I143" s="8" t="inlineStr"/>
+      <c r="J143" s="8" t="inlineStr"/>
     </row>
     <row r="144" ht="26" customHeight="1">
       <c r="A144" s="6" t="inlineStr">
         <is>
-          <t>Grupo Mais Empresas / Construções Mais</t>
+          <t>Grupo André Jordan</t>
         </is>
       </c>
       <c r="B144" s="8" t="inlineStr">
@@ -6269,30 +6261,34 @@
         </is>
       </c>
       <c r="C144" s="8" t="inlineStr"/>
-      <c r="D144" s="6" t="inlineStr"/>
+      <c r="D144" s="6" t="inlineStr">
+        <is>
+          <t>Gilberto Jordan (CEO desde 2009 · sucede a André Jordan, falecido 2024)</t>
+        </is>
+      </c>
       <c r="E144" s="6" t="inlineStr"/>
       <c r="F144" s="6" t="inlineStr"/>
       <c r="G144" s="6" t="inlineStr"/>
       <c r="H144" s="6" t="inlineStr">
         <is>
-          <t>grupomaisempresas.pt</t>
+          <t>andrejordangroup.pt</t>
         </is>
       </c>
       <c r="I144" s="8" t="inlineStr">
         <is>
-          <t>Leiria</t>
+          <t>Sintra</t>
         </is>
       </c>
       <c r="J144" s="8" t="inlineStr">
         <is>
-          <t>Leiria</t>
+          <t>Lisboa</t>
         </is>
       </c>
     </row>
     <row r="145" ht="26" customHeight="1">
       <c r="A145" s="6" t="inlineStr">
         <is>
-          <t>Grupo NB Portugal</t>
+          <t>Grupo AOC (Aníbal de Oliveira Cristina)</t>
         </is>
       </c>
       <c r="B145" s="8" t="inlineStr">
@@ -6303,32 +6299,28 @@
       <c r="C145" s="8" t="inlineStr"/>
       <c r="D145" s="6" t="inlineStr">
         <is>
-          <t>Ioav Blanche (presidente)</t>
+          <t>Aníbal Cristina (fundador, 1990)</t>
         </is>
       </c>
       <c r="E145" s="6" t="inlineStr"/>
       <c r="F145" s="6" t="inlineStr"/>
       <c r="G145" s="6" t="inlineStr"/>
-      <c r="H145" s="6" t="inlineStr">
-        <is>
-          <t>gruponbportugal.pt</t>
-        </is>
-      </c>
+      <c r="H145" s="6" t="inlineStr"/>
       <c r="I145" s="8" t="inlineStr">
         <is>
-          <t>Aveiro</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="J145" s="8" t="inlineStr">
         <is>
-          <t>Aveiro</t>
+          <t>Setúbal</t>
         </is>
       </c>
     </row>
     <row r="146" ht="26" customHeight="1">
       <c r="A146" s="6" t="inlineStr">
         <is>
-          <t>Grupo Pestana (Pestana Residences)</t>
+          <t>Grupo Mais Empresas / Construções Mais</t>
         </is>
       </c>
       <c r="B146" s="8" t="inlineStr">
@@ -6337,34 +6329,30 @@
         </is>
       </c>
       <c r="C146" s="8" t="inlineStr"/>
-      <c r="D146" s="6" t="inlineStr">
-        <is>
-          <t>Dionísio Pestana (Chairman/dono)</t>
-        </is>
-      </c>
+      <c r="D146" s="6" t="inlineStr"/>
       <c r="E146" s="6" t="inlineStr"/>
       <c r="F146" s="6" t="inlineStr"/>
       <c r="G146" s="6" t="inlineStr"/>
       <c r="H146" s="6" t="inlineStr">
         <is>
-          <t>pestana.com</t>
+          <t>grupomaisempresas.pt</t>
         </is>
       </c>
       <c r="I146" s="8" t="inlineStr">
         <is>
-          <t>Sines/Lagoa</t>
+          <t>Leiria</t>
         </is>
       </c>
       <c r="J146" s="8" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Leiria</t>
         </is>
       </c>
     </row>
     <row r="147" ht="26" customHeight="1">
       <c r="A147" s="6" t="inlineStr">
         <is>
-          <t>Hillside House Coimbra, Lda</t>
+          <t>Grupo NB Portugal</t>
         </is>
       </c>
       <c r="B147" s="8" t="inlineStr">
@@ -6373,18 +6361,22 @@
         </is>
       </c>
       <c r="C147" s="8" t="inlineStr"/>
-      <c r="D147" s="6" t="inlineStr"/>
+      <c r="D147" s="6" t="inlineStr">
+        <is>
+          <t>Ioav Blanche (presidente)</t>
+        </is>
+      </c>
       <c r="E147" s="6" t="inlineStr"/>
       <c r="F147" s="6" t="inlineStr"/>
       <c r="G147" s="6" t="inlineStr"/>
       <c r="H147" s="6" t="inlineStr">
         <is>
-          <t>hillside.pt</t>
+          <t>gruponbportugal.pt</t>
         </is>
       </c>
       <c r="I147" s="8" t="inlineStr">
         <is>
-          <t>Mealhada (projeto em Coimbra)</t>
+          <t>Aveiro</t>
         </is>
       </c>
       <c r="J147" s="8" t="inlineStr">
@@ -6396,7 +6388,7 @@
     <row r="148" ht="26" customHeight="1">
       <c r="A148" s="6" t="inlineStr">
         <is>
-          <t>Iconic Jeunesse, Unipessoal, Lda</t>
+          <t>Grupo Pestana (Pestana Residences)</t>
         </is>
       </c>
       <c r="B148" s="8" t="inlineStr">
@@ -6405,30 +6397,34 @@
         </is>
       </c>
       <c r="C148" s="8" t="inlineStr"/>
-      <c r="D148" s="6" t="inlineStr"/>
+      <c r="D148" s="6" t="inlineStr">
+        <is>
+          <t>Dionísio Pestana (Chairman/dono)</t>
+        </is>
+      </c>
       <c r="E148" s="6" t="inlineStr"/>
       <c r="F148" s="6" t="inlineStr"/>
       <c r="G148" s="6" t="inlineStr"/>
       <c r="H148" s="6" t="inlineStr">
         <is>
-          <t>zenithresidences.pt</t>
+          <t>pestana.com</t>
         </is>
       </c>
       <c r="I148" s="8" t="inlineStr">
         <is>
-          <t>Portimão</t>
+          <t>Sines/Lagoa</t>
         </is>
       </c>
       <c r="J148" s="8" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Setúbal</t>
         </is>
       </c>
     </row>
     <row r="149" ht="26" customHeight="1">
       <c r="A149" s="6" t="inlineStr">
         <is>
-          <t>Invesquart – Real Estate Promotor</t>
+          <t>Hillside House Coimbra, Lda</t>
         </is>
       </c>
       <c r="B149" s="8" t="inlineStr">
@@ -6441,22 +6437,26 @@
       <c r="E149" s="6" t="inlineStr"/>
       <c r="F149" s="6" t="inlineStr"/>
       <c r="G149" s="6" t="inlineStr"/>
-      <c r="H149" s="6" t="inlineStr"/>
+      <c r="H149" s="6" t="inlineStr">
+        <is>
+          <t>hillside.pt</t>
+        </is>
+      </c>
       <c r="I149" s="8" t="inlineStr">
         <is>
-          <t>Loulé (Quarteira)</t>
+          <t>Mealhada (projeto em Coimbra)</t>
         </is>
       </c>
       <c r="J149" s="8" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Aveiro</t>
         </is>
       </c>
     </row>
     <row r="150" ht="26" customHeight="1">
       <c r="A150" s="6" t="inlineStr">
         <is>
-          <t>Le Parc</t>
+          <t>Iconic Jeunesse, Unipessoal, Lda</t>
         </is>
       </c>
       <c r="B150" s="8" t="inlineStr">
@@ -6471,12 +6471,12 @@
       <c r="G150" s="6" t="inlineStr"/>
       <c r="H150" s="6" t="inlineStr">
         <is>
-          <t>leparc.pt</t>
+          <t>zenithresidences.pt</t>
         </is>
       </c>
       <c r="I150" s="8" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Portimão</t>
         </is>
       </c>
       <c r="J150" s="8" t="inlineStr">
@@ -6488,7 +6488,7 @@
     <row r="151" ht="26" customHeight="1">
       <c r="A151" s="6" t="inlineStr">
         <is>
-          <t>Lux Premium</t>
+          <t>Invesquart – Real Estate Promotor</t>
         </is>
       </c>
       <c r="B151" s="8" t="inlineStr">
@@ -6497,34 +6497,26 @@
         </is>
       </c>
       <c r="C151" s="8" t="inlineStr"/>
-      <c r="D151" s="6" t="inlineStr">
-        <is>
-          <t>Claude Berda (fundador)</t>
-        </is>
-      </c>
+      <c r="D151" s="6" t="inlineStr"/>
       <c r="E151" s="6" t="inlineStr"/>
       <c r="F151" s="6" t="inlineStr"/>
       <c r="G151" s="6" t="inlineStr"/>
-      <c r="H151" s="6" t="inlineStr">
-        <is>
-          <t>luxpremium.net</t>
-        </is>
-      </c>
+      <c r="H151" s="6" t="inlineStr"/>
       <c r="I151" s="8" t="inlineStr">
         <is>
-          <t>Coimbra</t>
+          <t>Loulé (Quarteira)</t>
         </is>
       </c>
       <c r="J151" s="8" t="inlineStr">
         <is>
-          <t>Coimbra</t>
+          <t>Faro</t>
         </is>
       </c>
     </row>
     <row r="152" ht="26" customHeight="1">
       <c r="A152" s="6" t="inlineStr">
         <is>
-          <t>MAJA Construções, S.A.</t>
+          <t>Le Parc</t>
         </is>
       </c>
       <c r="B152" s="8" t="inlineStr">
@@ -6533,18 +6525,18 @@
         </is>
       </c>
       <c r="C152" s="8" t="inlineStr"/>
-      <c r="D152" s="6" t="inlineStr">
-        <is>
-          <t>Manuel António e Jorge Almeida (fundadores, 1972)</t>
-        </is>
-      </c>
+      <c r="D152" s="6" t="inlineStr"/>
       <c r="E152" s="6" t="inlineStr"/>
       <c r="F152" s="6" t="inlineStr"/>
       <c r="G152" s="6" t="inlineStr"/>
-      <c r="H152" s="6" t="inlineStr"/>
+      <c r="H152" s="6" t="inlineStr">
+        <is>
+          <t>leparc.pt</t>
+        </is>
+      </c>
       <c r="I152" s="8" t="inlineStr">
         <is>
-          <t>Albufeira</t>
+          <t>Faro</t>
         </is>
       </c>
       <c r="J152" s="8" t="inlineStr">
@@ -6556,7 +6548,7 @@
     <row r="153" ht="26" customHeight="1">
       <c r="A153" s="6" t="inlineStr">
         <is>
-          <t>Mariano Investe – Empreendimentos Imobiliários</t>
+          <t>Lux Premium</t>
         </is>
       </c>
       <c r="B153" s="8" t="inlineStr">
@@ -6565,26 +6557,34 @@
         </is>
       </c>
       <c r="C153" s="8" t="inlineStr"/>
-      <c r="D153" s="6" t="inlineStr"/>
+      <c r="D153" s="6" t="inlineStr">
+        <is>
+          <t>Claude Berda (fundador)</t>
+        </is>
+      </c>
       <c r="E153" s="6" t="inlineStr"/>
       <c r="F153" s="6" t="inlineStr"/>
       <c r="G153" s="6" t="inlineStr"/>
-      <c r="H153" s="6" t="inlineStr"/>
+      <c r="H153" s="6" t="inlineStr">
+        <is>
+          <t>luxpremium.net</t>
+        </is>
+      </c>
       <c r="I153" s="8" t="inlineStr">
         <is>
-          <t>Santarém</t>
+          <t>Coimbra</t>
         </is>
       </c>
       <c r="J153" s="8" t="inlineStr">
         <is>
-          <t>Santarém</t>
+          <t>Coimbra</t>
         </is>
       </c>
     </row>
     <row r="154" ht="26" customHeight="1">
       <c r="A154" s="6" t="inlineStr">
         <is>
-          <t>Maven (Maven Invest)</t>
+          <t>MAJA Construções, S.A.</t>
         </is>
       </c>
       <c r="B154" s="8" t="inlineStr">
@@ -6595,32 +6595,28 @@
       <c r="C154" s="8" t="inlineStr"/>
       <c r="D154" s="6" t="inlineStr">
         <is>
-          <t>Yehonatan Gourvitch (CEO)</t>
+          <t>Manuel António e Jorge Almeida (fundadores, 1972)</t>
         </is>
       </c>
       <c r="E154" s="6" t="inlineStr"/>
       <c r="F154" s="6" t="inlineStr"/>
       <c r="G154" s="6" t="inlineStr"/>
-      <c r="H154" s="6" t="inlineStr">
-        <is>
-          <t>maveninvest.pt</t>
-        </is>
-      </c>
+      <c r="H154" s="6" t="inlineStr"/>
       <c r="I154" s="8" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Albufeira</t>
         </is>
       </c>
       <c r="J154" s="8" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Faro</t>
         </is>
       </c>
     </row>
     <row r="155" ht="26" customHeight="1">
       <c r="A155" s="6" t="inlineStr">
         <is>
-          <t>Máscarazul – Mediação Imobiliária, Lda</t>
+          <t>Mariano Investe – Empreendimentos Imobiliários</t>
         </is>
       </c>
       <c r="B155" s="8" t="inlineStr">
@@ -6636,19 +6632,19 @@
       <c r="H155" s="6" t="inlineStr"/>
       <c r="I155" s="8" t="inlineStr">
         <is>
-          <t>Albufeira</t>
+          <t>Santarém</t>
         </is>
       </c>
       <c r="J155" s="8" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Santarém</t>
         </is>
       </c>
     </row>
     <row r="156" ht="26" customHeight="1">
       <c r="A156" s="6" t="inlineStr">
         <is>
-          <t>Nova Atlantic</t>
+          <t>Maven (Maven Invest)</t>
         </is>
       </c>
       <c r="B156" s="8" t="inlineStr">
@@ -6659,28 +6655,32 @@
       <c r="C156" s="8" t="inlineStr"/>
       <c r="D156" s="6" t="inlineStr">
         <is>
-          <t>Matan Amitai (co-fundador)</t>
+          <t>Yehonatan Gourvitch (CEO)</t>
         </is>
       </c>
       <c r="E156" s="6" t="inlineStr"/>
       <c r="F156" s="6" t="inlineStr"/>
       <c r="G156" s="6" t="inlineStr"/>
-      <c r="H156" s="6" t="inlineStr"/>
+      <c r="H156" s="6" t="inlineStr">
+        <is>
+          <t>maveninvest.pt</t>
+        </is>
+      </c>
       <c r="I156" s="8" t="inlineStr">
         <is>
-          <t>Viana do Castelo</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="J156" s="8" t="inlineStr">
         <is>
-          <t>Viana do Castelo</t>
+          <t>Setúbal</t>
         </is>
       </c>
     </row>
     <row r="157" ht="26" customHeight="1">
       <c r="A157" s="6" t="inlineStr">
         <is>
-          <t>OCM Portugal (O'Connor Murphy)</t>
+          <t>Máscarazul – Mediação Imobiliária, Lda</t>
         </is>
       </c>
       <c r="B157" s="8" t="inlineStr">
@@ -6693,14 +6693,10 @@
       <c r="E157" s="6" t="inlineStr"/>
       <c r="F157" s="6" t="inlineStr"/>
       <c r="G157" s="6" t="inlineStr"/>
-      <c r="H157" s="6" t="inlineStr">
-        <is>
-          <t>oconnormurphy.ie</t>
-        </is>
-      </c>
+      <c r="H157" s="6" t="inlineStr"/>
       <c r="I157" s="8" t="inlineStr">
         <is>
-          <t>Olhão</t>
+          <t>Albufeira</t>
         </is>
       </c>
       <c r="J157" s="8" t="inlineStr">
@@ -6712,7 +6708,7 @@
     <row r="158" ht="26" customHeight="1">
       <c r="A158" s="6" t="inlineStr">
         <is>
-          <t>PATRIMOINIMMO PORTUGAL</t>
+          <t>Nova Atlantic</t>
         </is>
       </c>
       <c r="B158" s="8" t="inlineStr">
@@ -6721,26 +6717,30 @@
         </is>
       </c>
       <c r="C158" s="8" t="inlineStr"/>
-      <c r="D158" s="6" t="inlineStr"/>
+      <c r="D158" s="6" t="inlineStr">
+        <is>
+          <t>Matan Amitai (co-fundador)</t>
+        </is>
+      </c>
       <c r="E158" s="6" t="inlineStr"/>
       <c r="F158" s="6" t="inlineStr"/>
       <c r="G158" s="6" t="inlineStr"/>
       <c r="H158" s="6" t="inlineStr"/>
       <c r="I158" s="8" t="inlineStr">
         <is>
-          <t>Lagoa</t>
+          <t>Viana do Castelo</t>
         </is>
       </c>
       <c r="J158" s="8" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Viana do Castelo</t>
         </is>
       </c>
     </row>
     <row r="159" ht="26" customHeight="1">
       <c r="A159" s="6" t="inlineStr">
         <is>
-          <t>Pelicano – Investimento Imobiliário, S.A.</t>
+          <t>OCM Portugal (O'Connor Murphy)</t>
         </is>
       </c>
       <c r="B159" s="8" t="inlineStr">
@@ -6749,30 +6749,30 @@
         </is>
       </c>
       <c r="C159" s="8" t="inlineStr"/>
-      <c r="D159" s="6" t="inlineStr">
-        <is>
-          <t>Joaquim Da Cunha Mendes Duarte (Presidente) / Sergio Manuel Mendes Gomes (Administrador)</t>
-        </is>
-      </c>
+      <c r="D159" s="6" t="inlineStr"/>
       <c r="E159" s="6" t="inlineStr"/>
       <c r="F159" s="6" t="inlineStr"/>
       <c r="G159" s="6" t="inlineStr"/>
-      <c r="H159" s="6" t="inlineStr"/>
+      <c r="H159" s="6" t="inlineStr">
+        <is>
+          <t>oconnormurphy.ie</t>
+        </is>
+      </c>
       <c r="I159" s="8" t="inlineStr">
         <is>
-          <t>Palmela</t>
+          <t>Olhão</t>
         </is>
       </c>
       <c r="J159" s="8" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Faro</t>
         </is>
       </c>
     </row>
     <row r="160" ht="26" customHeight="1">
       <c r="A160" s="6" t="inlineStr">
         <is>
-          <t>Pensaplano</t>
+          <t>PATRIMOINIMMO PORTUGAL</t>
         </is>
       </c>
       <c r="B160" s="8" t="inlineStr">
@@ -6788,19 +6788,19 @@
       <c r="H160" s="6" t="inlineStr"/>
       <c r="I160" s="8" t="inlineStr">
         <is>
-          <t>Coimbra</t>
+          <t>Lagoa</t>
         </is>
       </c>
       <c r="J160" s="8" t="inlineStr">
         <is>
-          <t>Coimbra</t>
+          <t>Faro</t>
         </is>
       </c>
     </row>
     <row r="161" ht="26" customHeight="1">
       <c r="A161" s="6" t="inlineStr">
         <is>
-          <t>Portugal Slow Living</t>
+          <t>Pelicano – Investimento Imobiliário, S.A.</t>
         </is>
       </c>
       <c r="B161" s="8" t="inlineStr">
@@ -6809,14 +6809,18 @@
         </is>
       </c>
       <c r="C161" s="8" t="inlineStr"/>
-      <c r="D161" s="6" t="inlineStr"/>
+      <c r="D161" s="6" t="inlineStr">
+        <is>
+          <t>Joaquim Da Cunha Mendes Duarte (Presidente) / Sergio Manuel Mendes Gomes (Administrador)</t>
+        </is>
+      </c>
       <c r="E161" s="6" t="inlineStr"/>
       <c r="F161" s="6" t="inlineStr"/>
       <c r="G161" s="6" t="inlineStr"/>
       <c r="H161" s="6" t="inlineStr"/>
       <c r="I161" s="8" t="inlineStr">
         <is>
-          <t>Montijo</t>
+          <t>Palmela</t>
         </is>
       </c>
       <c r="J161" s="8" t="inlineStr">
@@ -6828,7 +6832,7 @@
     <row r="162" ht="26" customHeight="1">
       <c r="A162" s="6" t="inlineStr">
         <is>
-          <t>Rivage Properties</t>
+          <t>Pensaplano</t>
         </is>
       </c>
       <c r="B162" s="8" t="inlineStr">
@@ -6837,30 +6841,26 @@
         </is>
       </c>
       <c r="C162" s="8" t="inlineStr"/>
-      <c r="D162" s="6" t="inlineStr">
-        <is>
-          <t>João Ribeiro (CEO e fundador, com Jorge Duarte e Fernando Santos)</t>
-        </is>
-      </c>
+      <c r="D162" s="6" t="inlineStr"/>
       <c r="E162" s="6" t="inlineStr"/>
       <c r="F162" s="6" t="inlineStr"/>
       <c r="G162" s="6" t="inlineStr"/>
       <c r="H162" s="6" t="inlineStr"/>
       <c r="I162" s="8" t="inlineStr">
         <is>
-          <t>Gondomar</t>
+          <t>Coimbra</t>
         </is>
       </c>
       <c r="J162" s="8" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Coimbra</t>
         </is>
       </c>
     </row>
     <row r="163" ht="26" customHeight="1">
       <c r="A163" s="6" t="inlineStr">
         <is>
-          <t>Rodrigues &amp; Vermelho – Construções, S.A.</t>
+          <t>Portugal Slow Living</t>
         </is>
       </c>
       <c r="B163" s="8" t="inlineStr">
@@ -6869,34 +6869,26 @@
         </is>
       </c>
       <c r="C163" s="8" t="inlineStr"/>
-      <c r="D163" s="6" t="inlineStr">
-        <is>
-          <t>Celestino Vermelho Rodrigues (contacto)</t>
-        </is>
-      </c>
+      <c r="D163" s="6" t="inlineStr"/>
       <c r="E163" s="6" t="inlineStr"/>
       <c r="F163" s="6" t="inlineStr"/>
       <c r="G163" s="6" t="inlineStr"/>
-      <c r="H163" s="6" t="inlineStr">
-        <is>
-          <t>rodriguesevermelho.com</t>
-        </is>
-      </c>
+      <c r="H163" s="6" t="inlineStr"/>
       <c r="I163" s="8" t="inlineStr">
         <is>
-          <t>Lagos</t>
+          <t>Montijo</t>
         </is>
       </c>
       <c r="J163" s="8" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Setúbal</t>
         </is>
       </c>
     </row>
     <row r="164" ht="26" customHeight="1">
       <c r="A164" s="6" t="inlineStr">
         <is>
-          <t>SOLUM PROGRESS</t>
+          <t>Rivage Properties</t>
         </is>
       </c>
       <c r="B164" s="8" t="inlineStr">
@@ -6905,26 +6897,30 @@
         </is>
       </c>
       <c r="C164" s="8" t="inlineStr"/>
-      <c r="D164" s="6" t="inlineStr"/>
+      <c r="D164" s="6" t="inlineStr">
+        <is>
+          <t>João Ribeiro (CEO e fundador, com Jorge Duarte e Fernando Santos)</t>
+        </is>
+      </c>
       <c r="E164" s="6" t="inlineStr"/>
       <c r="F164" s="6" t="inlineStr"/>
       <c r="G164" s="6" t="inlineStr"/>
       <c r="H164" s="6" t="inlineStr"/>
       <c r="I164" s="8" t="inlineStr">
         <is>
-          <t>Coimbra</t>
+          <t>Gondomar</t>
         </is>
       </c>
       <c r="J164" s="8" t="inlineStr">
         <is>
-          <t>Coimbra</t>
+          <t>Porto</t>
         </is>
       </c>
     </row>
     <row r="165" ht="26" customHeight="1">
       <c r="A165" s="6" t="inlineStr">
         <is>
-          <t>Southshore Investments</t>
+          <t>Rodrigues &amp; Vermelho – Construções, S.A.</t>
         </is>
       </c>
       <c r="B165" s="8" t="inlineStr">
@@ -6933,30 +6929,34 @@
         </is>
       </c>
       <c r="C165" s="8" t="inlineStr"/>
-      <c r="D165" s="6" t="inlineStr"/>
+      <c r="D165" s="6" t="inlineStr">
+        <is>
+          <t>Celestino Vermelho Rodrigues (contacto)</t>
+        </is>
+      </c>
       <c r="E165" s="6" t="inlineStr"/>
       <c r="F165" s="6" t="inlineStr"/>
       <c r="G165" s="6" t="inlineStr"/>
       <c r="H165" s="6" t="inlineStr">
         <is>
-          <t>southshoreinvest.com</t>
+          <t>rodriguesevermelho.com</t>
         </is>
       </c>
       <c r="I165" s="8" t="inlineStr">
         <is>
-          <t>Almada</t>
+          <t>Lagos</t>
         </is>
       </c>
       <c r="J165" s="8" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Faro</t>
         </is>
       </c>
     </row>
     <row r="166" ht="26" customHeight="1">
       <c r="A166" s="6" t="inlineStr">
         <is>
-          <t>Terrace Benefit, Lda</t>
+          <t>SOLUM PROGRESS</t>
         </is>
       </c>
       <c r="B166" s="8" t="inlineStr">
@@ -6972,19 +6972,19 @@
       <c r="H166" s="6" t="inlineStr"/>
       <c r="I166" s="8" t="inlineStr">
         <is>
-          <t>Loulé (Quarteira)</t>
+          <t>Coimbra</t>
         </is>
       </c>
       <c r="J166" s="8" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Coimbra</t>
         </is>
       </c>
     </row>
     <row r="167" ht="26" customHeight="1">
       <c r="A167" s="6" t="inlineStr">
         <is>
-          <t>The Epic Group</t>
+          <t>Southshore Investments</t>
         </is>
       </c>
       <c r="B167" s="8" t="inlineStr">
@@ -6999,24 +6999,24 @@
       <c r="G167" s="6" t="inlineStr"/>
       <c r="H167" s="6" t="inlineStr">
         <is>
-          <t>valentavillas.com</t>
+          <t>southshoreinvest.com</t>
         </is>
       </c>
       <c r="I167" s="8" t="inlineStr">
         <is>
-          <t>Ílhavo</t>
+          <t>Almada</t>
         </is>
       </c>
       <c r="J167" s="8" t="inlineStr">
         <is>
-          <t>Aveiro</t>
+          <t>Setúbal</t>
         </is>
       </c>
     </row>
     <row r="168" ht="26" customHeight="1">
       <c r="A168" s="6" t="inlineStr">
         <is>
-          <t>Udra – Grupo San José</t>
+          <t>Terrace Benefit, Lda</t>
         </is>
       </c>
       <c r="B168" s="8" t="inlineStr">
@@ -7032,19 +7032,19 @@
       <c r="H168" s="6" t="inlineStr"/>
       <c r="I168" s="8" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Loulé (Quarteira)</t>
         </is>
       </c>
       <c r="J168" s="8" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Faro</t>
         </is>
       </c>
     </row>
     <row r="169" ht="26" customHeight="1">
       <c r="A169" s="6" t="inlineStr">
         <is>
-          <t>Urban Green Private (UGP)</t>
+          <t>The Epic Group</t>
         </is>
       </c>
       <c r="B169" s="8" t="inlineStr">
@@ -7053,34 +7053,30 @@
         </is>
       </c>
       <c r="C169" s="8" t="inlineStr"/>
-      <c r="D169" s="6" t="inlineStr">
-        <is>
-          <t>Thomas Coughlan (fundador)</t>
-        </is>
-      </c>
+      <c r="D169" s="6" t="inlineStr"/>
       <c r="E169" s="6" t="inlineStr"/>
       <c r="F169" s="6" t="inlineStr"/>
       <c r="G169" s="6" t="inlineStr"/>
       <c r="H169" s="6" t="inlineStr">
         <is>
-          <t>ugp.ie</t>
+          <t>valentavillas.com</t>
         </is>
       </c>
       <c r="I169" s="8" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Ílhavo</t>
         </is>
       </c>
       <c r="J169" s="8" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Aveiro</t>
         </is>
       </c>
     </row>
     <row r="170" ht="26" customHeight="1">
       <c r="A170" s="6" t="inlineStr">
         <is>
-          <t>Urban Office</t>
+          <t>Udra – Grupo San José</t>
         </is>
       </c>
       <c r="B170" s="8" t="inlineStr">
@@ -7093,26 +7089,22 @@
       <c r="E170" s="6" t="inlineStr"/>
       <c r="F170" s="6" t="inlineStr"/>
       <c r="G170" s="6" t="inlineStr"/>
-      <c r="H170" s="6" t="inlineStr">
-        <is>
-          <t>urbanoffice.pt</t>
-        </is>
-      </c>
+      <c r="H170" s="6" t="inlineStr"/>
       <c r="I170" s="8" t="inlineStr">
         <is>
-          <t>Torres Vedras</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="J170" s="8" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Setúbal</t>
         </is>
       </c>
     </row>
     <row r="171" ht="26" customHeight="1">
       <c r="A171" s="6" t="inlineStr">
         <is>
-          <t>Vale do Lobo Resort</t>
+          <t>Urban Green Private (UGP)</t>
         </is>
       </c>
       <c r="B171" s="8" t="inlineStr">
@@ -7121,18 +7113,22 @@
         </is>
       </c>
       <c r="C171" s="8" t="inlineStr"/>
-      <c r="D171" s="6" t="inlineStr"/>
+      <c r="D171" s="6" t="inlineStr">
+        <is>
+          <t>Thomas Coughlan (fundador)</t>
+        </is>
+      </c>
       <c r="E171" s="6" t="inlineStr"/>
       <c r="F171" s="6" t="inlineStr"/>
       <c r="G171" s="6" t="inlineStr"/>
       <c r="H171" s="6" t="inlineStr">
         <is>
-          <t>valedolobo.com</t>
+          <t>ugp.ie</t>
         </is>
       </c>
       <c r="I171" s="8" t="inlineStr">
         <is>
-          <t>Loulé</t>
+          <t>Faro</t>
         </is>
       </c>
       <c r="J171" s="8" t="inlineStr">
@@ -7144,7 +7140,7 @@
     <row r="172" ht="26" customHeight="1">
       <c r="A172" s="6" t="inlineStr">
         <is>
-          <t>Vila Galé</t>
+          <t>Urban Office</t>
         </is>
       </c>
       <c r="B172" s="8" t="inlineStr">
@@ -7159,15 +7155,79 @@
       <c r="G172" s="6" t="inlineStr"/>
       <c r="H172" s="6" t="inlineStr">
         <is>
+          <t>urbanoffice.pt</t>
+        </is>
+      </c>
+      <c r="I172" s="8" t="inlineStr">
+        <is>
+          <t>Torres Vedras</t>
+        </is>
+      </c>
+      <c r="J172" s="8" t="inlineStr">
+        <is>
+          <t>Lisboa</t>
+        </is>
+      </c>
+    </row>
+    <row r="173" ht="26" customHeight="1">
+      <c r="A173" s="6" t="inlineStr">
+        <is>
+          <t>Vale do Lobo Resort</t>
+        </is>
+      </c>
+      <c r="B173" s="8" t="inlineStr">
+        <is>
+          <t>Nao</t>
+        </is>
+      </c>
+      <c r="C173" s="8" t="inlineStr"/>
+      <c r="D173" s="6" t="inlineStr"/>
+      <c r="E173" s="6" t="inlineStr"/>
+      <c r="F173" s="6" t="inlineStr"/>
+      <c r="G173" s="6" t="inlineStr"/>
+      <c r="H173" s="6" t="inlineStr">
+        <is>
+          <t>valedolobo.com</t>
+        </is>
+      </c>
+      <c r="I173" s="8" t="inlineStr">
+        <is>
+          <t>Loulé</t>
+        </is>
+      </c>
+      <c r="J173" s="8" t="inlineStr">
+        <is>
+          <t>Faro</t>
+        </is>
+      </c>
+    </row>
+    <row r="174" ht="26" customHeight="1">
+      <c r="A174" s="6" t="inlineStr">
+        <is>
+          <t>Vila Galé</t>
+        </is>
+      </c>
+      <c r="B174" s="8" t="inlineStr">
+        <is>
+          <t>Nao</t>
+        </is>
+      </c>
+      <c r="C174" s="8" t="inlineStr"/>
+      <c r="D174" s="6" t="inlineStr"/>
+      <c r="E174" s="6" t="inlineStr"/>
+      <c r="F174" s="6" t="inlineStr"/>
+      <c r="G174" s="6" t="inlineStr"/>
+      <c r="H174" s="6" t="inlineStr">
+        <is>
           <t>vilagale.com</t>
         </is>
       </c>
-      <c r="I172" s="8" t="inlineStr">
+      <c r="I174" s="8" t="inlineStr">
         <is>
           <t>Golegã</t>
         </is>
       </c>
-      <c r="J172" s="8" t="inlineStr">
+      <c r="J174" s="8" t="inlineStr">
         <is>
           <t>Santarém</t>
         </is>
@@ -7224,16 +7284,16 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E88" r:id="rId47"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E89" r:id="rId48"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E90" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E109" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E110" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E111" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E112" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E113" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E114" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E115" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E116" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E117" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E118" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E111" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E112" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E113" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E114" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E115" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E116" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E117" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E118" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E119" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E120" r:id="rId59"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
@@ -7274,7 +7334,7 @@
         </is>
       </c>
       <c r="B2" s="11" t="n">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="3">
@@ -7294,7 +7354,7 @@
         </is>
       </c>
       <c r="B4" s="11" t="n">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="5">
@@ -7334,7 +7394,7 @@
         </is>
       </c>
       <c r="B8" s="11" t="n">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="9">

</xml_diff>